<commit_message>
Dashboard update Tue 04/28/2026 22:27
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9CAA7158-3300-436D-A5B9-5DB5B1790BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9CD99F63-21D9-441A-9548-BC1A36FEBB46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-52875" yWindow="2205" windowWidth="50145" windowHeight="27570" xr2:uid="{D7C1C753-0486-404B-8498-9D23BF02A5A7}"/>
+    <workbookView xWindow="0" yWindow="4830" windowWidth="57810" windowHeight="27570" xr2:uid="{D7C1C753-0486-404B-8498-9D23BF02A5A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3474,7 +3474,7 @@
         <v>45108</v>
       </c>
       <c r="Y38" s="17">
-        <v>46265</v>
+        <v>46996</v>
       </c>
       <c r="Z38" s="24" t="s">
         <v>90</v>
@@ -3483,7 +3483,7 @@
         <v>91</v>
       </c>
       <c r="AB38" s="20">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AC38" s="20"/>
       <c r="AD38" s="23"/>
@@ -13243,7 +13243,7 @@
         <v>12.615643397813288</v>
       </c>
       <c r="R183" s="14">
-        <v>5000</v>
+        <v>3750</v>
       </c>
       <c r="S183" s="29">
         <v>45066</v>
@@ -13252,7 +13252,7 @@
         <v>45108</v>
       </c>
       <c r="U183" s="29">
-        <v>46265</v>
+        <v>46996</v>
       </c>
       <c r="V183" s="14">
         <v>0</v>
@@ -13312,7 +13312,7 @@
         <v>25.231286795626577</v>
       </c>
       <c r="R184" s="14">
-        <v>10000</v>
+        <v>7500</v>
       </c>
       <c r="S184" s="17">
         <v>45066</v>
@@ -13321,7 +13321,7 @@
         <v>45108</v>
       </c>
       <c r="U184" s="29">
-        <v>46265</v>
+        <v>46996</v>
       </c>
       <c r="V184" s="14">
         <v>0</v>
@@ -13381,7 +13381,7 @@
         <v>26.24053826745164</v>
       </c>
       <c r="R185" s="14">
-        <v>10400</v>
+        <v>7800</v>
       </c>
       <c r="S185" s="17">
         <v>45066</v>
@@ -13390,7 +13390,7 @@
         <v>45108</v>
       </c>
       <c r="U185" s="29">
-        <v>46265</v>
+        <v>46996</v>
       </c>
       <c r="V185" s="14">
         <v>0</v>
@@ -13450,7 +13450,7 @@
         <v>27.249789739276704</v>
       </c>
       <c r="R186" s="14">
-        <v>10800</v>
+        <v>8100</v>
       </c>
       <c r="S186" s="17">
         <v>45066</v>
@@ -13459,7 +13459,7 @@
         <v>45108</v>
       </c>
       <c r="U186" s="29">
-        <v>46265</v>
+        <v>46996</v>
       </c>
       <c r="V186" s="14">
         <v>0</v>
@@ -13467,142 +13467,142 @@
       <c r="W186" s="14"/>
     </row>
     <row r="187" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A187" s="30" t="s">
+      <c r="A187" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B187" s="30" t="s">
+      <c r="B187" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C187" s="30">
+      <c r="C187" s="5">
         <v>5</v>
       </c>
-      <c r="D187" s="30" t="s">
+      <c r="D187" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E187" s="30" t="s">
-        <v>110</v>
-      </c>
-      <c r="F187" s="30">
+      <c r="E187" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F187" s="5">
         <v>5</v>
       </c>
-      <c r="G187" s="31">
+      <c r="G187" s="17">
         <v>46266</v>
       </c>
-      <c r="H187" s="31">
+      <c r="H187" s="17">
         <v>46630</v>
       </c>
-      <c r="I187" s="32">
+      <c r="I187" s="11">
         <v>0.11111111111111116</v>
       </c>
-      <c r="J187" s="33">
+      <c r="J187" s="14">
         <v>3000</v>
       </c>
-      <c r="K187" s="42">
+      <c r="K187" s="41">
         <v>36000</v>
       </c>
-      <c r="L187" s="30" t="s">
+      <c r="L187" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="M187" s="34">
+      <c r="M187" s="7">
         <v>1189</v>
       </c>
-      <c r="N187" s="32">
+      <c r="N187" s="11">
         <v>0.39</v>
       </c>
-      <c r="O187" s="32">
+      <c r="O187" s="11">
         <v>0.39</v>
       </c>
-      <c r="P187" s="32">
-        <v>0</v>
-      </c>
-      <c r="Q187" s="33">
+      <c r="P187" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q187" s="14">
         <v>30.277544154751894</v>
       </c>
-      <c r="R187" s="33">
-        <v>12000</v>
-      </c>
-      <c r="S187" s="31">
+      <c r="R187" s="14">
+        <v>9000</v>
+      </c>
+      <c r="S187" s="17">
         <v>45066</v>
       </c>
-      <c r="T187" s="31">
+      <c r="T187" s="17">
         <v>45108</v>
       </c>
       <c r="U187" s="29">
-        <v>46265</v>
-      </c>
-      <c r="V187" s="33">
-        <v>0</v>
-      </c>
-      <c r="W187" s="33"/>
+        <v>46996</v>
+      </c>
+      <c r="V187" s="14">
+        <v>0</v>
+      </c>
+      <c r="W187" s="14"/>
     </row>
     <row r="188" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A188" s="30" t="s">
+      <c r="A188" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B188" s="30" t="s">
+      <c r="B188" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C188" s="30">
+      <c r="C188" s="5">
         <v>5</v>
       </c>
-      <c r="D188" s="30" t="s">
+      <c r="D188" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E188" s="30" t="s">
-        <v>110</v>
-      </c>
-      <c r="F188" s="30">
+      <c r="E188" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F188" s="5">
         <v>6</v>
       </c>
-      <c r="G188" s="31">
+      <c r="G188" s="17">
         <v>46631</v>
       </c>
-      <c r="H188" s="31">
+      <c r="H188" s="17">
         <v>46996</v>
       </c>
-      <c r="I188" s="32">
+      <c r="I188" s="11">
         <v>3.3333333333333437E-2</v>
       </c>
-      <c r="J188" s="33">
+      <c r="J188" s="14">
         <v>3100</v>
       </c>
-      <c r="K188" s="42">
+      <c r="K188" s="41">
         <v>37200</v>
       </c>
-      <c r="L188" s="30" t="s">
+      <c r="L188" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="M188" s="34">
+      <c r="M188" s="7">
         <v>1189</v>
       </c>
-      <c r="N188" s="32">
+      <c r="N188" s="11">
         <v>0.39</v>
       </c>
-      <c r="O188" s="32">
+      <c r="O188" s="11">
         <v>0.39</v>
       </c>
-      <c r="P188" s="32">
-        <v>0</v>
-      </c>
-      <c r="Q188" s="33">
+      <c r="P188" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q188" s="14">
         <v>31.286795626576957</v>
       </c>
-      <c r="R188" s="33">
-        <v>12400</v>
-      </c>
-      <c r="S188" s="31">
+      <c r="R188" s="14">
+        <v>9300</v>
+      </c>
+      <c r="S188" s="17">
         <v>45066</v>
       </c>
-      <c r="T188" s="31">
+      <c r="T188" s="17">
         <v>45108</v>
       </c>
       <c r="U188" s="29">
-        <v>46265</v>
-      </c>
-      <c r="V188" s="33">
-        <v>0</v>
-      </c>
-      <c r="W188" s="33"/>
+        <v>46996</v>
+      </c>
+      <c r="V188" s="14">
+        <v>0</v>
+      </c>
+      <c r="W188" s="14"/>
     </row>
     <row r="189" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A189" s="35" t="s">
@@ -13657,7 +13657,7 @@
         <v>33.30529857022708</v>
       </c>
       <c r="R189" s="38">
-        <v>13200</v>
+        <v>9900</v>
       </c>
       <c r="S189" s="36">
         <v>45066</v>
@@ -13666,7 +13666,7 @@
         <v>45108</v>
       </c>
       <c r="U189" s="29">
-        <v>46265</v>
+        <v>46996</v>
       </c>
       <c r="V189" s="38">
         <v>0</v>
@@ -13726,7 +13726,7 @@
         <v>34.314550042052147</v>
       </c>
       <c r="R190" s="38">
-        <v>13600</v>
+        <v>10200</v>
       </c>
       <c r="S190" s="36">
         <v>45066</v>
@@ -13735,7 +13735,7 @@
         <v>45108</v>
       </c>
       <c r="U190" s="29">
-        <v>46265</v>
+        <v>46996</v>
       </c>
       <c r="V190" s="38">
         <v>0</v>

</xml_diff>

<commit_message>
Dashboard update Tue 04/28/2026 22:36
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9CD99F63-21D9-441A-9548-BC1A36FEBB46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F3578BC-0C73-4DD0-BC9D-FEEE74D61272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="4830" windowWidth="57810" windowHeight="27570" xr2:uid="{D7C1C753-0486-404B-8498-9D23BF02A5A7}"/>
+    <workbookView xWindow="495" yWindow="2100" windowWidth="57810" windowHeight="27570" xr2:uid="{D7C1C753-0486-404B-8498-9D23BF02A5A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3897,7 +3897,7 @@
         <v>2</v>
       </c>
       <c r="G48" s="17">
-        <v>45383</v>
+        <v>45748</v>
       </c>
       <c r="H48" s="17">
         <v>46112</v>
@@ -3966,7 +3966,7 @@
         <v>3</v>
       </c>
       <c r="G49" s="17">
-        <v>45383</v>
+        <v>46113</v>
       </c>
       <c r="H49" s="17">
         <v>46477</v>
@@ -4035,7 +4035,7 @@
         <v>4</v>
       </c>
       <c r="G50" s="17">
-        <v>45383</v>
+        <v>46478</v>
       </c>
       <c r="H50" s="17">
         <v>46843</v>
@@ -4104,7 +4104,7 @@
         <v>5</v>
       </c>
       <c r="G51" s="17">
-        <v>45383</v>
+        <v>46844</v>
       </c>
       <c r="H51" s="17">
         <v>47208</v>
@@ -4173,7 +4173,7 @@
         <v>6</v>
       </c>
       <c r="G52" s="17">
-        <v>45383</v>
+        <v>47209</v>
       </c>
       <c r="H52" s="17">
         <v>47573</v>
@@ -4242,7 +4242,7 @@
         <v>7</v>
       </c>
       <c r="G53" s="17">
-        <v>45383</v>
+        <v>47574</v>
       </c>
       <c r="H53" s="17">
         <v>47938</v>
@@ -4311,7 +4311,7 @@
         <v>8</v>
       </c>
       <c r="G54" s="17">
-        <v>45383</v>
+        <v>47939</v>
       </c>
       <c r="H54" s="17">
         <v>48304</v>
@@ -4380,7 +4380,7 @@
         <v>9</v>
       </c>
       <c r="G55" s="17">
-        <v>45383</v>
+        <v>48305</v>
       </c>
       <c r="H55" s="17">
         <v>48669</v>
@@ -4449,7 +4449,7 @@
         <v>10</v>
       </c>
       <c r="G56" s="17">
-        <v>45383</v>
+        <v>48670</v>
       </c>
       <c r="H56" s="17">
         <v>49034</v>
@@ -4518,7 +4518,7 @@
         <v>11</v>
       </c>
       <c r="G57" s="31">
-        <v>45383</v>
+        <v>49035</v>
       </c>
       <c r="H57" s="31">
         <v>49399</v>
@@ -4587,7 +4587,7 @@
         <v>12</v>
       </c>
       <c r="G58" s="31">
-        <v>45383</v>
+        <v>49400</v>
       </c>
       <c r="H58" s="31">
         <v>49765</v>
@@ -4656,7 +4656,7 @@
         <v>13</v>
       </c>
       <c r="G59" s="31">
-        <v>45383</v>
+        <v>49766</v>
       </c>
       <c r="H59" s="31">
         <v>50130</v>
@@ -4725,7 +4725,7 @@
         <v>14</v>
       </c>
       <c r="G60" s="31">
-        <v>45383</v>
+        <v>50131</v>
       </c>
       <c r="H60" s="31">
         <v>50495</v>
@@ -4794,7 +4794,7 @@
         <v>15</v>
       </c>
       <c r="G61" s="31">
-        <v>45383</v>
+        <v>50496</v>
       </c>
       <c r="H61" s="31">
         <v>50860</v>
@@ -4863,7 +4863,7 @@
         <v>16</v>
       </c>
       <c r="G62" s="36">
-        <v>45383</v>
+        <v>50861</v>
       </c>
       <c r="H62" s="36">
         <v>51226</v>
@@ -4932,7 +4932,7 @@
         <v>17</v>
       </c>
       <c r="G63" s="36">
-        <v>45383</v>
+        <v>51227</v>
       </c>
       <c r="H63" s="36">
         <v>51591</v>
@@ -5001,7 +5001,7 @@
         <v>18</v>
       </c>
       <c r="G64" s="36">
-        <v>45383</v>
+        <v>51592</v>
       </c>
       <c r="H64" s="36">
         <v>51956</v>
@@ -5070,7 +5070,7 @@
         <v>19</v>
       </c>
       <c r="G65" s="36">
-        <v>45383</v>
+        <v>51957</v>
       </c>
       <c r="H65" s="36">
         <v>52321</v>
@@ -5139,7 +5139,7 @@
         <v>20</v>
       </c>
       <c r="G66" s="36">
-        <v>45383</v>
+        <v>52322</v>
       </c>
       <c r="H66" s="36">
         <v>52687</v>

</xml_diff>

<commit_message>
Dashboard update Tue 05/12/2026  6:33
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A71F962-7529-46C5-A092-563D7194B201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C428DD5D-2C05-4E61-AD93-DED4470F1432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1560" windowWidth="69795" windowHeight="29895" xr2:uid="{F2AD7EB6-AB81-41AA-B966-6E7976896F31}"/>
+    <workbookView xWindow="0" yWindow="2505" windowWidth="57810" windowHeight="29895" xr2:uid="{8A02A6E0-EEF3-4C0D-8740-D5447D1DA22A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2099" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2143" uniqueCount="191">
   <si>
     <t>Building</t>
   </si>
@@ -191,7 +191,7 @@
     <t>Select Tenant:</t>
   </si>
   <si>
-    <t>114 Central_207_Westfield Education Association</t>
+    <t xml:space="preserve">114 Central_202_Tang Pacific LLC D/BA ARSA </t>
   </si>
   <si>
     <t>EJS Westfield Toybox, LLC d/b/a Learning Express</t>
@@ -203,7 +203,7 @@
     <t>Tenant</t>
   </si>
   <si>
-    <t>Westfield Education Association</t>
+    <t xml:space="preserve">Tang Pacific LLC D/BA ARSA </t>
   </si>
   <si>
     <t>Reves Smoothie Bar, LLC d/b/a Reves Cafe</t>
@@ -240,9 +240,6 @@
   </si>
   <si>
     <t>Mths Left</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tang Pacific LLC D/BA ARSA </t>
   </si>
   <si>
     <t>Annual Variable</t>
@@ -297,6 +294,9 @@
   </si>
   <si>
     <t>Clauses</t>
+  </si>
+  <si>
+    <t>Westfield Education Association</t>
   </si>
   <si>
     <t>One-Two Year</t>
@@ -392,6 +392,9 @@
     <t>Two 5-Year 3% Annual Inc</t>
   </si>
   <si>
+    <t>Option_1</t>
+  </si>
+  <si>
     <t>Longo Architects &amp; Associates, LLC</t>
   </si>
   <si>
@@ -411,9 +414,6 @@
   </si>
   <si>
     <t>Two 5-Year 7.5% Jump then Flat</t>
-  </si>
-  <si>
-    <t>Option_1</t>
   </si>
   <si>
     <t>George's Appliance, LLC</t>
@@ -593,9 +593,6 @@
     <t>114 Central_201_Ashford - Schael, LLC</t>
   </si>
   <si>
-    <t xml:space="preserve">114 Central_202_Tang Pacific LLC D/BA ARSA </t>
-  </si>
-  <si>
     <t>114 Central_203_Rentokil North America dba Terminix</t>
   </si>
   <si>
@@ -609,6 +606,9 @@
   </si>
   <si>
     <t>114 Central_206_Dave Rossi Photography, LLC</t>
+  </si>
+  <si>
+    <t>114 Central_207_Westfield Education Association</t>
   </si>
   <si>
     <t>114 Central_208_SRD Capital Management, LLC</t>
@@ -1349,7 +1349,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AD14F0B-91B4-4C6E-A4EC-64272DDBC3CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{444630EB-1CC8-4A81-9DDA-D3668A4DB0D3}">
   <dimension ref="A1:AW260"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1429,7 +1429,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="7">
-        <v>130000</v>
+        <v>130001</v>
       </c>
       <c r="C2" s="8">
         <v>4894</v>
@@ -1951,7 +1951,7 @@
         <v>58</v>
       </c>
       <c r="AT13" s="27">
-        <v>793</v>
+        <v>607</v>
       </c>
     </row>
     <row r="14" spans="1:48" x14ac:dyDescent="0.25">
@@ -2060,7 +2060,7 @@
         <v>60</v>
       </c>
       <c r="AT14" s="28">
-        <v>47483</v>
+        <v>46507</v>
       </c>
     </row>
     <row r="15" spans="1:48" x14ac:dyDescent="0.25">
@@ -2163,13 +2163,13 @@
         <v>65</v>
       </c>
       <c r="AL15" s="22">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="AS15" s="23" t="s">
         <v>66</v>
       </c>
       <c r="AT15" s="30">
-        <v>44.333333333333336</v>
+        <v>11.766666666666667</v>
       </c>
     </row>
     <row r="16" spans="1:48" x14ac:dyDescent="0.25">
@@ -2180,7 +2180,7 @@
         <v>202</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>62</v>
@@ -2247,7 +2247,7 @@
         <v>46507</v>
       </c>
       <c r="Z16" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA16" s="18">
         <v>46327</v>
@@ -2257,10 +2257,10 @@
       </c>
       <c r="AC16" s="19"/>
       <c r="AD16" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE16" s="16" t="s">
         <v>69</v>
-      </c>
-      <c r="AE16" s="16" t="s">
-        <v>70</v>
       </c>
       <c r="AF16" s="13">
         <v>0</v>
@@ -2281,10 +2281,10 @@
         <v>27</v>
       </c>
       <c r="AS16" s="23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AT16" s="31">
-        <v>17.402269861286253</v>
+        <v>20.757825370675452</v>
       </c>
     </row>
     <row r="17" spans="1:49" x14ac:dyDescent="0.25">
@@ -2295,7 +2295,7 @@
         <v>203</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>62</v>
@@ -2371,7 +2371,7 @@
       <c r="AC17" s="19"/>
       <c r="AD17" s="32"/>
       <c r="AE17" s="32" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AF17" s="13">
         <v>0</v>
@@ -2389,19 +2389,19 @@
         <v>58</v>
       </c>
       <c r="AL17" s="27">
-        <v>793</v>
+        <v>607</v>
       </c>
       <c r="AM17" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="AN17" s="31">
+        <v>1050</v>
+      </c>
+      <c r="AS17" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="AN17" s="31">
-        <v>0</v>
-      </c>
-      <c r="AS17" s="23" t="s">
-        <v>75</v>
-      </c>
       <c r="AT17" s="33">
-        <v>6.448465135190079E-2</v>
+        <v>4.9359625940231758E-2</v>
       </c>
     </row>
     <row r="18" spans="1:49" x14ac:dyDescent="0.25">
@@ -2412,7 +2412,7 @@
         <v>204</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>62</v>
@@ -2470,13 +2470,13 @@
         <v>-10.571254319983737</v>
       </c>
       <c r="W18" s="16">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="X18" s="16">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="Y18" s="16">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="Z18" s="17"/>
       <c r="AA18" s="18" t="s">
@@ -2502,19 +2502,19 @@
         <v>19</v>
       </c>
       <c r="AL18" s="34">
-        <v>0.16121162837975198</v>
+        <v>0.12339906485057939</v>
       </c>
       <c r="AM18" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="AN18" s="34">
+        <v>0</v>
+      </c>
+      <c r="AS18" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="AN18" s="34">
-        <v>0</v>
-      </c>
-      <c r="AS18" s="23" t="s">
-        <v>78</v>
-      </c>
       <c r="AT18" s="35">
-        <v>47303</v>
+        <v>46327</v>
       </c>
     </row>
     <row r="19" spans="1:49" x14ac:dyDescent="0.25">
@@ -2525,7 +2525,7 @@
         <v>205</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>62</v>
@@ -2614,22 +2614,22 @@
         <v>1225</v>
       </c>
       <c r="AK19" s="26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="AL19" s="34">
-        <v>6.448465135190079E-2</v>
+        <v>4.9359625940231758E-2</v>
       </c>
       <c r="AM19" s="26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AN19" s="34">
-        <v>6.448465135190079E-2</v>
+        <v>4.9359625940231758E-2</v>
       </c>
       <c r="AS19" s="23" t="s">
         <v>35</v>
       </c>
       <c r="AT19" s="36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:49" x14ac:dyDescent="0.25">
@@ -2640,7 +2640,7 @@
         <v>206</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>62</v>
@@ -2707,7 +2707,7 @@
         <v>47968</v>
       </c>
       <c r="Z20" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA20" s="18">
         <v>46417</v>
@@ -2717,7 +2717,7 @@
       </c>
       <c r="AC20" s="19"/>
       <c r="AD20" s="16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AE20" s="16"/>
       <c r="AF20" s="13">
@@ -2733,22 +2733,22 @@
         <v>1465</v>
       </c>
       <c r="AK20" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="AL20" s="28">
+        <v>41640</v>
+      </c>
+      <c r="AM20" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="AL20" s="28">
-        <v>39520</v>
-      </c>
-      <c r="AM20" s="26" t="s">
+      <c r="AN20" s="34">
+        <v>-4.9359625940231758E-2</v>
+      </c>
+      <c r="AS20" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="AN20" s="34">
-        <v>-6.448465135190079E-2</v>
-      </c>
-      <c r="AS20" s="23" t="s">
-        <v>85</v>
-      </c>
       <c r="AT20" s="27" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:49" x14ac:dyDescent="0.25">
@@ -2759,7 +2759,7 @@
         <v>207</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>62</v>
@@ -2853,7 +2853,7 @@
         <v>87</v>
       </c>
       <c r="AL21" s="28">
-        <v>39520</v>
+        <v>41640</v>
       </c>
       <c r="AM21" s="26" t="s">
         <v>88</v>
@@ -2968,19 +2968,19 @@
         <v>60</v>
       </c>
       <c r="AL22" s="38">
-        <v>47483</v>
+        <v>46507</v>
       </c>
       <c r="AM22" s="26" t="s">
         <v>66</v>
       </c>
       <c r="AN22" s="30">
-        <v>44.333333333333336</v>
+        <v>11.766666666666667</v>
       </c>
       <c r="AS22" s="23" t="s">
         <v>66</v>
       </c>
       <c r="AT22" s="39">
-        <v>4.9333333333333336</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="23" spans="1:49" x14ac:dyDescent="0.25">
@@ -3361,7 +3361,7 @@
         <v>108</v>
       </c>
       <c r="AR26" s="56" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AS26" s="56" t="s">
         <v>26</v>
@@ -3472,43 +3472,43 @@
         <v>0</v>
       </c>
       <c r="AK27" s="22" t="s">
-        <v>113</v>
-      </c>
-      <c r="AL27" s="58">
-        <v>1</v>
-      </c>
-      <c r="AM27" s="28">
-        <v>46023</v>
-      </c>
-      <c r="AN27" s="28">
-        <v>46387</v>
-      </c>
-      <c r="AO27" s="34">
-        <v>0</v>
-      </c>
-      <c r="AP27" s="59">
-        <v>1150</v>
-      </c>
-      <c r="AQ27" s="60">
-        <v>13800</v>
-      </c>
-      <c r="AR27" s="59">
-        <v>17.402269861286253</v>
-      </c>
-      <c r="AS27" s="60">
-        <v>6.448465135190079E-2</v>
-      </c>
-      <c r="AT27" s="60">
-        <v>0</v>
+        <v>94</v>
+      </c>
+      <c r="AL27" s="58" t="s">
+        <v>94</v>
+      </c>
+      <c r="AM27" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN27" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO27" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP27" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ27" s="60" t="s">
+        <v>94</v>
+      </c>
+      <c r="AR27" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="AS27" s="60" t="s">
+        <v>94</v>
+      </c>
+      <c r="AT27" s="60" t="s">
+        <v>94</v>
       </c>
       <c r="AU27" s="60" t="s">
         <v>94</v>
       </c>
       <c r="AV27" s="61" t="s">
-        <v>27</v>
-      </c>
-      <c r="AW27" s="59">
-        <v>0</v>
+        <v>94</v>
+      </c>
+      <c r="AW27" s="59" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="28" spans="1:49" x14ac:dyDescent="0.25">
@@ -3557,34 +3557,34 @@
         <v>113</v>
       </c>
       <c r="AL28" s="62">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM28" s="63">
-        <v>46388</v>
+        <v>46143</v>
       </c>
       <c r="AN28" s="63">
-        <v>46752</v>
+        <v>46507</v>
       </c>
       <c r="AO28" s="64">
-        <v>0.47826086956521729</v>
+        <v>1.0960334029227556</v>
       </c>
       <c r="AP28" s="65">
-        <v>1700</v>
+        <v>1050</v>
       </c>
       <c r="AQ28" s="66">
-        <v>20400</v>
+        <v>12600</v>
       </c>
       <c r="AR28" s="65">
-        <v>25.725094577553595</v>
+        <v>20.757825370675452</v>
       </c>
       <c r="AS28" s="66">
-        <v>6.448465135190079E-2</v>
+        <v>4.9359625940231758E-2</v>
       </c>
       <c r="AT28" s="66">
-        <v>1700</v>
-      </c>
-      <c r="AU28" s="66">
-        <v>1700</v>
+        <v>1050</v>
+      </c>
+      <c r="AU28" s="66" t="s">
+        <v>94</v>
       </c>
       <c r="AV28" s="67" t="s">
         <v>27</v>
@@ -3694,37 +3694,37 @@
         <v>16933.333333333332</v>
       </c>
       <c r="AK29" s="22" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="AL29" s="58">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AM29" s="28">
-        <v>46753</v>
+        <v>46508</v>
       </c>
       <c r="AN29" s="28">
-        <v>47118</v>
+        <v>46873</v>
       </c>
       <c r="AO29" s="34">
-        <v>3.0000000000000027E-2</v>
+        <v>1.2380952380952381</v>
       </c>
       <c r="AP29" s="59">
-        <v>1751</v>
+        <v>1300</v>
       </c>
       <c r="AQ29" s="60">
-        <v>21012</v>
+        <v>15600</v>
       </c>
       <c r="AR29" s="59">
-        <v>26.4968474148802</v>
+        <v>25.7001647446458</v>
       </c>
       <c r="AS29" s="60">
-        <v>6.448465135190079E-2</v>
+        <v>4.9359625940231758E-2</v>
       </c>
       <c r="AT29" s="60">
-        <v>1751</v>
+        <v>1300</v>
       </c>
       <c r="AU29" s="60">
-        <v>51</v>
+        <v>250</v>
       </c>
       <c r="AV29" s="61" t="s">
         <v>27</v>
@@ -3741,7 +3741,7 @@
         <v>2</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>62</v>
@@ -3750,7 +3750,7 @@
         <v>2</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="6">
@@ -3811,7 +3811,7 @@
         <v>0.05</v>
       </c>
       <c r="AA30" s="32" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AB30" s="19">
         <v>2</v>
@@ -3832,43 +3832,43 @@
         <v>8747.9166666666661</v>
       </c>
       <c r="AK30" s="22" t="s">
-        <v>113</v>
-      </c>
-      <c r="AL30" s="62">
-        <v>4</v>
-      </c>
-      <c r="AM30" s="63">
-        <v>47119</v>
-      </c>
-      <c r="AN30" s="63">
-        <v>47483</v>
-      </c>
-      <c r="AO30" s="64">
-        <v>3.0000000000000027E-2</v>
-      </c>
-      <c r="AP30" s="65">
-        <v>1803.53</v>
-      </c>
-      <c r="AQ30" s="66">
-        <v>21642.36</v>
-      </c>
-      <c r="AR30" s="65">
-        <v>27.291752837326609</v>
-      </c>
-      <c r="AS30" s="66">
-        <v>6.448465135190079E-2</v>
-      </c>
-      <c r="AT30" s="66">
-        <v>1803.53</v>
-      </c>
-      <c r="AU30" s="66">
-        <v>52.529999999999973</v>
+        <v>94</v>
+      </c>
+      <c r="AL30" s="62" t="s">
+        <v>94</v>
+      </c>
+      <c r="AM30" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN30" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO30" s="64" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP30" s="65" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ30" s="66" t="s">
+        <v>94</v>
+      </c>
+      <c r="AR30" s="65" t="s">
+        <v>94</v>
+      </c>
+      <c r="AS30" s="66" t="s">
+        <v>94</v>
+      </c>
+      <c r="AT30" s="66" t="s">
+        <v>94</v>
+      </c>
+      <c r="AU30" s="66" t="s">
+        <v>94</v>
       </c>
       <c r="AV30" s="67" t="s">
-        <v>27</v>
-      </c>
-      <c r="AW30" s="65">
-        <v>0</v>
+        <v>94</v>
+      </c>
+      <c r="AW30" s="65" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="31" spans="1:49" x14ac:dyDescent="0.25">
@@ -3879,16 +3879,16 @@
         <v>3</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E31" s="6">
         <v>3</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G31" s="6"/>
       <c r="H31" s="6">
@@ -3949,7 +3949,7 @@
         <v>0</v>
       </c>
       <c r="AA31" s="32" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AB31" s="19"/>
       <c r="AC31" s="19"/>
@@ -3968,43 +3968,43 @@
         <v>0</v>
       </c>
       <c r="AK31" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="AL31" s="58">
-        <v>5</v>
-      </c>
-      <c r="AM31" s="28">
-        <v>47484</v>
-      </c>
-      <c r="AN31" s="28">
-        <v>47848</v>
-      </c>
-      <c r="AO31" s="34">
-        <v>5.0000092411363495E-2</v>
-      </c>
-      <c r="AP31" s="59">
-        <v>1893.7066666666667</v>
-      </c>
-      <c r="AQ31" s="60">
-        <v>22724.48</v>
-      </c>
-      <c r="AR31" s="59">
-        <v>28.656343001261032</v>
-      </c>
-      <c r="AS31" s="60">
-        <v>6.448465135190079E-2</v>
-      </c>
-      <c r="AT31" s="60">
-        <v>1893.7066666666667</v>
-      </c>
-      <c r="AU31" s="60">
-        <v>90.176666666666733</v>
+        <v>94</v>
+      </c>
+      <c r="AL31" s="58" t="s">
+        <v>94</v>
+      </c>
+      <c r="AM31" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN31" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO31" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP31" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ31" s="60" t="s">
+        <v>94</v>
+      </c>
+      <c r="AR31" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="AS31" s="60" t="s">
+        <v>94</v>
+      </c>
+      <c r="AT31" s="60" t="s">
+        <v>94</v>
+      </c>
+      <c r="AU31" s="60" t="s">
+        <v>94</v>
       </c>
       <c r="AV31" s="61" t="s">
-        <v>27</v>
-      </c>
-      <c r="AW31" s="59">
-        <v>0</v>
+        <v>94</v>
+      </c>
+      <c r="AW31" s="59" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:49" x14ac:dyDescent="0.25">
@@ -4024,7 +4024,7 @@
         <v>3</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G32" s="6"/>
       <c r="H32" s="6">
@@ -4100,43 +4100,43 @@
         <v>0</v>
       </c>
       <c r="AK32" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="AL32" s="62">
-        <v>6</v>
-      </c>
-      <c r="AM32" s="63">
-        <v>47849</v>
-      </c>
-      <c r="AN32" s="63">
-        <v>48213</v>
-      </c>
-      <c r="AO32" s="64">
-        <v>3.0002006646576707E-2</v>
-      </c>
-      <c r="AP32" s="65">
-        <v>1950.5216666666665</v>
-      </c>
-      <c r="AQ32" s="66">
-        <v>23406.26</v>
-      </c>
-      <c r="AR32" s="65">
-        <v>29.516090794451447</v>
-      </c>
-      <c r="AS32" s="66">
-        <v>6.448465135190079E-2</v>
-      </c>
-      <c r="AT32" s="66">
-        <v>1950.5216666666665</v>
-      </c>
-      <c r="AU32" s="66">
-        <v>56.814999999999827</v>
+        <v>94</v>
+      </c>
+      <c r="AL32" s="62" t="s">
+        <v>94</v>
+      </c>
+      <c r="AM32" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN32" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO32" s="64" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP32" s="65" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ32" s="66" t="s">
+        <v>94</v>
+      </c>
+      <c r="AR32" s="65" t="s">
+        <v>94</v>
+      </c>
+      <c r="AS32" s="66" t="s">
+        <v>94</v>
+      </c>
+      <c r="AT32" s="66" t="s">
+        <v>94</v>
+      </c>
+      <c r="AU32" s="66" t="s">
+        <v>94</v>
       </c>
       <c r="AV32" s="67" t="s">
-        <v>27</v>
-      </c>
-      <c r="AW32" s="65">
-        <v>0</v>
+        <v>94</v>
+      </c>
+      <c r="AW32" s="65" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="33" spans="1:49" x14ac:dyDescent="0.25">
@@ -6468,25 +6468,25 @@
         <v>113</v>
       </c>
       <c r="AL55" s="58">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AM55" s="28">
-        <v>46023</v>
+        <v>45778</v>
       </c>
       <c r="AN55" s="28">
-        <v>47483</v>
+        <v>46507</v>
       </c>
       <c r="AO55" s="59">
-        <v>1150</v>
+        <v>958</v>
       </c>
       <c r="AP55" s="60">
-        <v>13800</v>
+        <v>11496</v>
       </c>
       <c r="AQ55" s="59">
-        <v>1803.53</v>
+        <v>1050</v>
       </c>
       <c r="AR55" s="60">
-        <v>21642.36</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="56" spans="1:49" x14ac:dyDescent="0.25">
@@ -6561,25 +6561,25 @@
         <v>160</v>
       </c>
       <c r="AL56" s="58">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM56" s="28">
-        <v>47484</v>
+        <v>46508</v>
       </c>
       <c r="AN56" s="28">
-        <v>48213</v>
+        <v>46873</v>
       </c>
       <c r="AO56" s="59">
-        <v>1893.7066666666667</v>
+        <v>1300</v>
       </c>
       <c r="AP56" s="60">
-        <v>22724.48</v>
+        <v>15600</v>
       </c>
       <c r="AQ56" s="59">
-        <v>1950.5216666666665</v>
+        <v>1300</v>
       </c>
       <c r="AR56" s="60">
-        <v>23406.26</v>
+        <v>15600</v>
       </c>
     </row>
     <row r="57" spans="1:49" x14ac:dyDescent="0.25">
@@ -6596,7 +6596,7 @@
         <v>114</v>
       </c>
       <c r="E57" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F57" s="73">
         <v>11</v>
@@ -6689,7 +6689,7 @@
         <v>114</v>
       </c>
       <c r="E58" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F58" s="73">
         <v>12</v>
@@ -6782,7 +6782,7 @@
         <v>114</v>
       </c>
       <c r="E59" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F59" s="73">
         <v>13</v>
@@ -6851,7 +6851,7 @@
         <v>114</v>
       </c>
       <c r="E60" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F60" s="73">
         <v>14</v>
@@ -6920,7 +6920,7 @@
         <v>114</v>
       </c>
       <c r="E61" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F61" s="73">
         <v>15</v>
@@ -7400,7 +7400,7 @@
         <v>2</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>113</v>
@@ -7469,7 +7469,7 @@
         <v>2</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E69" s="6" t="s">
         <v>113</v>
@@ -7538,7 +7538,7 @@
         <v>2</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>113</v>
@@ -7607,7 +7607,7 @@
         <v>2</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E71" s="6" t="s">
         <v>113</v>
@@ -7745,7 +7745,7 @@
         <v>3</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E73" s="6" t="s">
         <v>113</v>
@@ -7814,7 +7814,7 @@
         <v>3</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>113</v>
@@ -7883,7 +7883,7 @@
         <v>3</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E75" s="6" t="s">
         <v>113</v>
@@ -7952,7 +7952,7 @@
         <v>3</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>113</v>
@@ -8021,7 +8021,7 @@
         <v>3</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>113</v>
@@ -8090,7 +8090,7 @@
         <v>3</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>113</v>
@@ -8159,7 +8159,7 @@
         <v>3</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E79" s="6" t="s">
         <v>113</v>
@@ -8228,7 +8228,7 @@
         <v>3</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>113</v>
@@ -8297,7 +8297,7 @@
         <v>3</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E81" s="6" t="s">
         <v>113</v>
@@ -8366,7 +8366,7 @@
         <v>3</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>113</v>
@@ -8435,7 +8435,7 @@
         <v>3</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E83" s="6" t="s">
         <v>113</v>
@@ -8504,7 +8504,7 @@
         <v>3</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>113</v>
@@ -8573,7 +8573,7 @@
         <v>3</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E85" s="6" t="s">
         <v>113</v>
@@ -8642,7 +8642,7 @@
         <v>3</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>113</v>
@@ -10301,7 +10301,7 @@
         <v>95</v>
       </c>
       <c r="E110" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F110" s="73">
         <v>11</v>
@@ -10370,7 +10370,7 @@
         <v>95</v>
       </c>
       <c r="E111" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F111" s="73">
         <v>12</v>
@@ -10439,7 +10439,7 @@
         <v>95</v>
       </c>
       <c r="E112" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F112" s="73">
         <v>13</v>
@@ -10508,7 +10508,7 @@
         <v>95</v>
       </c>
       <c r="E113" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F113" s="73">
         <v>14</v>
@@ -10577,7 +10577,7 @@
         <v>95</v>
       </c>
       <c r="E114" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F114" s="73">
         <v>15</v>
@@ -11060,7 +11060,7 @@
         <v>100</v>
       </c>
       <c r="E121" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F121" s="73">
         <v>6</v>
@@ -11129,7 +11129,7 @@
         <v>100</v>
       </c>
       <c r="E122" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F122" s="73">
         <v>7</v>
@@ -11198,7 +11198,7 @@
         <v>100</v>
       </c>
       <c r="E123" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F123" s="73">
         <v>8</v>
@@ -11267,7 +11267,7 @@
         <v>100</v>
       </c>
       <c r="E124" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F124" s="73">
         <v>9</v>
@@ -11336,7 +11336,7 @@
         <v>100</v>
       </c>
       <c r="E125" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F125" s="73">
         <v>10</v>
@@ -14232,7 +14232,7 @@
         <v>131</v>
       </c>
       <c r="E167" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F167" s="73">
         <v>11</v>
@@ -14301,7 +14301,7 @@
         <v>131</v>
       </c>
       <c r="E168" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F168" s="73">
         <v>12</v>
@@ -14370,7 +14370,7 @@
         <v>131</v>
       </c>
       <c r="E169" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F169" s="73">
         <v>13</v>
@@ -14439,7 +14439,7 @@
         <v>131</v>
       </c>
       <c r="E170" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F170" s="73">
         <v>14</v>
@@ -14508,7 +14508,7 @@
         <v>131</v>
       </c>
       <c r="E171" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F171" s="73">
         <v>15</v>
@@ -16992,7 +16992,7 @@
         <v>55</v>
       </c>
       <c r="E207" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F207" s="73">
         <v>7</v>
@@ -17061,7 +17061,7 @@
         <v>55</v>
       </c>
       <c r="E208" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F208" s="73">
         <v>8</v>
@@ -17130,7 +17130,7 @@
         <v>55</v>
       </c>
       <c r="E209" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F209" s="73">
         <v>9</v>
@@ -17199,7 +17199,7 @@
         <v>55</v>
       </c>
       <c r="E210" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F210" s="73">
         <v>10</v>
@@ -17268,7 +17268,7 @@
         <v>55</v>
       </c>
       <c r="E211" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F211" s="73">
         <v>11</v>
@@ -18360,7 +18360,7 @@
     </row>
     <row r="227" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A227" s="6" t="s">
-        <v>184</v>
+        <v>50</v>
       </c>
       <c r="B227" s="6" t="s">
         <v>6</v>
@@ -18369,7 +18369,7 @@
         <v>202</v>
       </c>
       <c r="D227" s="6" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="E227" s="6" t="s">
         <v>113</v>
@@ -18429,7 +18429,7 @@
     </row>
     <row r="228" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A228" s="6" t="s">
-        <v>184</v>
+        <v>50</v>
       </c>
       <c r="B228" s="6" t="s">
         <v>6</v>
@@ -18438,7 +18438,7 @@
         <v>202</v>
       </c>
       <c r="D228" s="6" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="E228" s="6" t="s">
         <v>113</v>
@@ -18498,7 +18498,7 @@
     </row>
     <row r="229" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A229" s="73" t="s">
-        <v>184</v>
+        <v>50</v>
       </c>
       <c r="B229" s="73" t="s">
         <v>6</v>
@@ -18507,10 +18507,10 @@
         <v>202</v>
       </c>
       <c r="D229" s="73" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="E229" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F229" s="73">
         <v>1</v>
@@ -18636,7 +18636,7 @@
     </row>
     <row r="231" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A231" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B231" s="6" t="s">
         <v>6</v>
@@ -18645,7 +18645,7 @@
         <v>203</v>
       </c>
       <c r="D231" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E231" s="6" t="s">
         <v>113</v>
@@ -18705,7 +18705,7 @@
     </row>
     <row r="232" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A232" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B232" s="6" t="s">
         <v>6</v>
@@ -18714,7 +18714,7 @@
         <v>203</v>
       </c>
       <c r="D232" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E232" s="6" t="s">
         <v>113</v>
@@ -18774,7 +18774,7 @@
     </row>
     <row r="233" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A233" s="73" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B233" s="73" t="s">
         <v>6</v>
@@ -18783,10 +18783,10 @@
         <v>203</v>
       </c>
       <c r="D233" s="73" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E233" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F233" s="73">
         <v>3</v>
@@ -18843,7 +18843,7 @@
     </row>
     <row r="234" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A234" s="78" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B234" s="78" t="s">
         <v>6</v>
@@ -18852,7 +18852,7 @@
         <v>203</v>
       </c>
       <c r="D234" s="78" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E234" s="78" t="s">
         <v>163</v>
@@ -18981,7 +18981,7 @@
     </row>
     <row r="236" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A236" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B236" s="6" t="s">
         <v>6</v>
@@ -18990,7 +18990,7 @@
         <v>204</v>
       </c>
       <c r="D236" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E236" s="6" t="s">
         <v>113</v>
@@ -18999,10 +18999,10 @@
         <v>1</v>
       </c>
       <c r="G236" s="93">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="H236" s="93">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="I236" s="10">
         <v>0</v>
@@ -19035,13 +19035,13 @@
         <v>0</v>
       </c>
       <c r="S236" s="70">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="T236" s="70">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="U236" s="70">
-        <v>46153</v>
+        <v>46154</v>
       </c>
       <c r="V236" s="13">
         <v>0</v>
@@ -19119,7 +19119,7 @@
     </row>
     <row r="238" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A238" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B238" s="6" t="s">
         <v>6</v>
@@ -19128,7 +19128,7 @@
         <v>205</v>
       </c>
       <c r="D238" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E238" s="6" t="s">
         <v>113</v>
@@ -19188,7 +19188,7 @@
     </row>
     <row r="239" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A239" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B239" s="6" t="s">
         <v>6</v>
@@ -19197,7 +19197,7 @@
         <v>205</v>
       </c>
       <c r="D239" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E239" s="6" t="s">
         <v>113</v>
@@ -19257,7 +19257,7 @@
     </row>
     <row r="240" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A240" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B240" s="6" t="s">
         <v>6</v>
@@ -19266,7 +19266,7 @@
         <v>205</v>
       </c>
       <c r="D240" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E240" s="6" t="s">
         <v>113</v>
@@ -19395,7 +19395,7 @@
     </row>
     <row r="242" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A242" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B242" s="6" t="s">
         <v>6</v>
@@ -19464,7 +19464,7 @@
     </row>
     <row r="243" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A243" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B243" s="6" t="s">
         <v>6</v>
@@ -19533,7 +19533,7 @@
     </row>
     <row r="244" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A244" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B244" s="6" t="s">
         <v>6</v>
@@ -19671,7 +19671,7 @@
     </row>
     <row r="246" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A246" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B246" s="6" t="s">
         <v>6</v>
@@ -19680,7 +19680,7 @@
         <v>206</v>
       </c>
       <c r="D246" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E246" s="6" t="s">
         <v>113</v>
@@ -19740,7 +19740,7 @@
     </row>
     <row r="247" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A247" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B247" s="6" t="s">
         <v>6</v>
@@ -19749,7 +19749,7 @@
         <v>206</v>
       </c>
       <c r="D247" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E247" s="6" t="s">
         <v>113</v>
@@ -19811,7 +19811,7 @@
     </row>
     <row r="248" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A248" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B248" s="6" t="s">
         <v>6</v>
@@ -19820,7 +19820,7 @@
         <v>206</v>
       </c>
       <c r="D248" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E248" s="6" t="s">
         <v>113</v>
@@ -19882,7 +19882,7 @@
     </row>
     <row r="249" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A249" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B249" s="6" t="s">
         <v>6</v>
@@ -19891,7 +19891,7 @@
         <v>206</v>
       </c>
       <c r="D249" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E249" s="6" t="s">
         <v>113</v>
@@ -19953,7 +19953,7 @@
     </row>
     <row r="250" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A250" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B250" s="6" t="s">
         <v>6</v>
@@ -19962,7 +19962,7 @@
         <v>206</v>
       </c>
       <c r="D250" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E250" s="6" t="s">
         <v>113</v>
@@ -20024,7 +20024,7 @@
     </row>
     <row r="251" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A251" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B251" s="6" t="s">
         <v>6</v>
@@ -20033,7 +20033,7 @@
         <v>206</v>
       </c>
       <c r="D251" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E251" s="6" t="s">
         <v>113</v>
@@ -20164,7 +20164,7 @@
     </row>
     <row r="253" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A253" s="6" t="s">
-        <v>50</v>
+        <v>189</v>
       </c>
       <c r="B253" s="6" t="s">
         <v>6</v>
@@ -20173,7 +20173,7 @@
         <v>207</v>
       </c>
       <c r="D253" s="6" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="E253" s="6" t="s">
         <v>113</v>
@@ -20233,7 +20233,7 @@
     </row>
     <row r="254" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A254" s="6" t="s">
-        <v>50</v>
+        <v>189</v>
       </c>
       <c r="B254" s="6" t="s">
         <v>6</v>
@@ -20242,7 +20242,7 @@
         <v>207</v>
       </c>
       <c r="D254" s="6" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="E254" s="6" t="s">
         <v>113</v>
@@ -20302,7 +20302,7 @@
     </row>
     <row r="255" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A255" s="6" t="s">
-        <v>50</v>
+        <v>189</v>
       </c>
       <c r="B255" s="6" t="s">
         <v>6</v>
@@ -20311,7 +20311,7 @@
         <v>207</v>
       </c>
       <c r="D255" s="6" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="E255" s="6" t="s">
         <v>113</v>
@@ -20371,7 +20371,7 @@
     </row>
     <row r="256" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A256" s="6" t="s">
-        <v>50</v>
+        <v>189</v>
       </c>
       <c r="B256" s="6" t="s">
         <v>6</v>
@@ -20380,7 +20380,7 @@
         <v>207</v>
       </c>
       <c r="D256" s="6" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="E256" s="6" t="s">
         <v>113</v>
@@ -20440,7 +20440,7 @@
     </row>
     <row r="257" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A257" s="73" t="s">
-        <v>50</v>
+        <v>189</v>
       </c>
       <c r="B257" s="73" t="s">
         <v>6</v>
@@ -20449,10 +20449,10 @@
         <v>207</v>
       </c>
       <c r="D257" s="73" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="E257" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F257" s="73">
         <v>5</v>
@@ -20509,7 +20509,7 @@
     </row>
     <row r="258" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A258" s="73" t="s">
-        <v>50</v>
+        <v>189</v>
       </c>
       <c r="B258" s="73" t="s">
         <v>6</v>
@@ -20518,10 +20518,10 @@
         <v>207</v>
       </c>
       <c r="D258" s="73" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="E258" s="73" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F258" s="73">
         <v>6</v>

</xml_diff>

<commit_message>
Dashboard update Tue 05/12/2026  6:43
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C428DD5D-2C05-4E61-AD93-DED4470F1432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{43564DC1-F923-4227-99BD-35898DD8D923}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2505" windowWidth="57810" windowHeight="29895" xr2:uid="{8A02A6E0-EEF3-4C0D-8740-D5447D1DA22A}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="57810" windowHeight="29895" xr2:uid="{98642A8E-0764-40C3-B15E-624F75792EAD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2143" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2171" uniqueCount="192">
   <si>
     <t>Building</t>
   </si>
@@ -203,9 +203,6 @@
     <t>Tenant</t>
   </si>
   <si>
-    <t xml:space="preserve">Tang Pacific LLC D/BA ARSA </t>
-  </si>
-  <si>
     <t>Reves Smoothie Bar, LLC d/b/a Reves Cafe</t>
   </si>
   <si>
@@ -240,6 +237,9 @@
   </si>
   <si>
     <t>Mths Left</t>
+  </si>
+  <si>
+    <t>Tang Pacific LLC D/BA ARSA</t>
   </si>
   <si>
     <t>Annual Variable</t>
@@ -380,9 +380,6 @@
     <t>Easement</t>
   </si>
   <si>
-    <t>Original</t>
-  </si>
-  <si>
     <t>HDR HOLDINGS LLC D/B/A WONDER</t>
   </si>
   <si>
@@ -390,9 +387,6 @@
   </si>
   <si>
     <t>Two 5-Year 3% Annual Inc</t>
-  </si>
-  <si>
-    <t>Option_1</t>
   </si>
   <si>
     <t>Longo Architects &amp; Associates, LLC</t>
@@ -494,6 +488,9 @@
     <t>36 South_1_HDR HOLDINGS LLC D/B/A WONDER</t>
   </si>
   <si>
+    <t>Original</t>
+  </si>
+  <si>
     <t>LEASE OPTIONS SUMMARY</t>
   </si>
   <si>
@@ -522,6 +519,9 @@
   </si>
   <si>
     <t>Option 1</t>
+  </si>
+  <si>
+    <t>Option_1</t>
   </si>
   <si>
     <t>Option 2</t>
@@ -578,19 +578,22 @@
     <t>1280 Springfield_7_Alan DiEsso</t>
   </si>
   <si>
-    <t>114 Central_1_Nabig Sakr</t>
+    <t>114 Central_102_Nabig Sakr</t>
   </si>
   <si>
-    <t>114 Central_2_EJS Westfield Toybox, LLC d/b/a Learning Express</t>
+    <t>114 Central_104_EJS Westfield Toybox, LLC d/b/a Learning Express</t>
   </si>
   <si>
-    <t>114 Central_3_Reves Smoothie Bar, LLC d/b/a Reves Cafe</t>
+    <t>114 Central_106_Reves Smoothie Bar, LLC d/b/a Reves Cafe</t>
   </si>
   <si>
-    <t>114 Central_4_Luna Wireless</t>
+    <t>114 Central_108_Luna Wireless</t>
   </si>
   <si>
     <t>114 Central_201_Ashford - Schael, LLC</t>
+  </si>
+  <si>
+    <t>114 Central_202_Tang Pacific LLC D/BA ARSA</t>
   </si>
   <si>
     <t>114 Central_203_Rentokil North America dba Terminix</t>
@@ -1349,7 +1352,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{444630EB-1CC8-4A81-9DDA-D3668A4DB0D3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01BBE3BE-0B5E-41B0-9D35-E128E88B66BC}">
   <dimension ref="A1:AW260"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1626,7 +1629,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="6">
-        <v>1</v>
+        <v>102</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>44</v>
@@ -1739,7 +1742,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="6">
-        <v>2</v>
+        <v>104</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>51</v>
@@ -1837,8 +1840,8 @@
       <c r="AS12" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="AT12" s="22" t="s">
-        <v>54</v>
+      <c r="AT12" s="22" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="13" spans="1:48" x14ac:dyDescent="0.25">
@@ -1846,10 +1849,10 @@
         <v>6</v>
       </c>
       <c r="B13" s="6">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>45</v>
@@ -1916,7 +1919,7 @@
         <v>46810</v>
       </c>
       <c r="Z13" s="17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AA13" s="18">
         <v>46565</v>
@@ -1927,7 +1930,7 @@
       <c r="AC13" s="19"/>
       <c r="AD13" s="16"/>
       <c r="AE13" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AF13" s="13">
         <v>11.637681159420289</v>
@@ -1944,14 +1947,14 @@
       <c r="AK13" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="AL13" s="22" t="s">
-        <v>54</v>
+      <c r="AL13" s="22" t="e">
+        <v>#N/A</v>
       </c>
       <c r="AS13" s="23" t="s">
-        <v>58</v>
-      </c>
-      <c r="AT13" s="27">
-        <v>607</v>
+        <v>57</v>
+      </c>
+      <c r="AT13" s="27" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="14" spans="1:48" x14ac:dyDescent="0.25">
@@ -1959,10 +1962,10 @@
         <v>6</v>
       </c>
       <c r="B14" s="6">
-        <v>4</v>
+        <v>108</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>45</v>
@@ -2053,14 +2056,14 @@
       <c r="AK14" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="AL14" s="22" t="s">
-        <v>6</v>
+      <c r="AL14" s="22" t="e">
+        <v>#N/A</v>
       </c>
       <c r="AS14" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AT14" s="28">
-        <v>46507</v>
+        <v>59</v>
+      </c>
+      <c r="AT14" s="28" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="15" spans="1:48" x14ac:dyDescent="0.25">
@@ -2071,16 +2074,16 @@
         <v>201</v>
       </c>
       <c r="C15" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="E15" s="6">
         <v>2</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G15" s="6"/>
       <c r="H15" s="6">
@@ -2145,7 +2148,7 @@
       <c r="AC15" s="19"/>
       <c r="AD15" s="16"/>
       <c r="AE15" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AF15" s="13">
         <v>0</v>
@@ -2160,16 +2163,16 @@
         <v>1632.5</v>
       </c>
       <c r="AK15" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="AL15" s="22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="AS15" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="AL15" s="22">
-        <v>202</v>
-      </c>
-      <c r="AS15" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="AT15" s="30">
-        <v>11.766666666666667</v>
+      <c r="AT15" s="30" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="16" spans="1:48" x14ac:dyDescent="0.25">
@@ -2180,16 +2183,16 @@
         <v>202</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E16" s="6">
         <v>2</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G16" s="6"/>
       <c r="H16" s="6">
@@ -2277,14 +2280,14 @@
       <c r="AK16" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="AL16" s="22" t="s">
-        <v>27</v>
+      <c r="AL16" s="22" t="e">
+        <v>#N/A</v>
       </c>
       <c r="AS16" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="AT16" s="31">
-        <v>20.757825370675452</v>
+      <c r="AT16" s="31" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="17" spans="1:49" x14ac:dyDescent="0.25">
@@ -2298,13 +2301,13 @@
         <v>71</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E17" s="6">
         <v>2</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G17" s="6"/>
       <c r="H17" s="6">
@@ -2386,22 +2389,22 @@
         <v>1555</v>
       </c>
       <c r="AK17" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="AL17" s="27">
-        <v>607</v>
+        <v>57</v>
+      </c>
+      <c r="AL17" s="27" t="e">
+        <v>#N/A</v>
       </c>
       <c r="AM17" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="AN17" s="31">
-        <v>1050</v>
+      <c r="AN17" s="31" t="e">
+        <v>#N/A</v>
       </c>
       <c r="AS17" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="AT17" s="33">
-        <v>4.9359625940231758E-2</v>
+      <c r="AT17" s="33" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="18" spans="1:49" x14ac:dyDescent="0.25">
@@ -2415,13 +2418,13 @@
         <v>75</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E18" s="6">
         <v>2</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G18" s="6"/>
       <c r="H18" s="6">
@@ -2501,20 +2504,20 @@
       <c r="AK18" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="AL18" s="34">
-        <v>0.12339906485057939</v>
+      <c r="AL18" s="34" t="e">
+        <v>#N/A</v>
       </c>
       <c r="AM18" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="AN18" s="34">
-        <v>0</v>
+      <c r="AN18" s="34" t="s">
+        <v>68</v>
       </c>
       <c r="AS18" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="AT18" s="35">
-        <v>46327</v>
+      <c r="AT18" s="35" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="19" spans="1:49" x14ac:dyDescent="0.25">
@@ -2528,13 +2531,13 @@
         <v>78</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E19" s="6">
         <v>2</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G19" s="6"/>
       <c r="H19" s="6">
@@ -2616,14 +2619,14 @@
       <c r="AK19" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="AL19" s="34">
-        <v>4.9359625940231758E-2</v>
+      <c r="AL19" s="34" t="e">
+        <v>#N/A</v>
       </c>
       <c r="AM19" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="AN19" s="34">
-        <v>4.9359625940231758E-2</v>
+      <c r="AN19" s="34" t="s">
+        <v>68</v>
       </c>
       <c r="AS19" s="23" t="s">
         <v>35</v>
@@ -2643,13 +2646,13 @@
         <v>80</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E20" s="6">
         <v>2</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G20" s="6"/>
       <c r="H20" s="6">
@@ -2735,20 +2738,20 @@
       <c r="AK20" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="AL20" s="28">
-        <v>41640</v>
+      <c r="AL20" s="28" t="e">
+        <v>#N/A</v>
       </c>
       <c r="AM20" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="AN20" s="34">
-        <v>-4.9359625940231758E-2</v>
+      <c r="AN20" s="34" t="e">
+        <v>#VALUE!</v>
       </c>
       <c r="AS20" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="AT20" s="27" t="s">
-        <v>69</v>
+      <c r="AT20" s="27" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="21" spans="1:49" x14ac:dyDescent="0.25">
@@ -2762,13 +2765,13 @@
         <v>85</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E21" s="6">
         <v>2</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G21" s="6"/>
       <c r="H21" s="6">
@@ -2852,14 +2855,14 @@
       <c r="AK21" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="AL21" s="28">
-        <v>41640</v>
+      <c r="AL21" s="28" t="e">
+        <v>#N/A</v>
       </c>
       <c r="AM21" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="AN21" s="31">
-        <v>0</v>
+      <c r="AN21" s="31" t="e">
+        <v>#N/A</v>
       </c>
       <c r="AS21" s="23" t="s">
         <v>89</v>
@@ -2879,13 +2882,13 @@
         <v>90</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E22" s="6">
         <v>2</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G22" s="6"/>
       <c r="H22" s="6">
@@ -2965,19 +2968,19 @@
         <v>680</v>
       </c>
       <c r="AK22" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL22" s="38">
-        <v>46507</v>
+        <v>59</v>
+      </c>
+      <c r="AL22" s="38" t="e">
+        <v>#N/A</v>
       </c>
       <c r="AM22" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="AN22" s="30">
-        <v>11.766666666666667</v>
+        <v>65</v>
+      </c>
+      <c r="AN22" s="30" t="e">
+        <v>#N/A</v>
       </c>
       <c r="AS22" s="23" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AT22" s="39">
         <v>4.9000000000000004</v>
@@ -2994,13 +2997,13 @@
         <v>91</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E23" s="6">
         <v>2</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G23" s="6"/>
       <c r="H23" s="6">
@@ -3554,43 +3557,43 @@
       </c>
       <c r="AI28" s="45"/>
       <c r="AK28" s="22" t="s">
-        <v>113</v>
-      </c>
-      <c r="AL28" s="62">
-        <v>1</v>
-      </c>
-      <c r="AM28" s="63">
-        <v>46143</v>
-      </c>
-      <c r="AN28" s="63">
-        <v>46507</v>
-      </c>
-      <c r="AO28" s="64">
-        <v>1.0960334029227556</v>
-      </c>
-      <c r="AP28" s="65">
-        <v>1050</v>
-      </c>
-      <c r="AQ28" s="66">
-        <v>12600</v>
-      </c>
-      <c r="AR28" s="65">
-        <v>20.757825370675452</v>
-      </c>
-      <c r="AS28" s="66">
-        <v>4.9359625940231758E-2</v>
-      </c>
-      <c r="AT28" s="66">
-        <v>1050</v>
+        <v>94</v>
+      </c>
+      <c r="AL28" s="62" t="s">
+        <v>94</v>
+      </c>
+      <c r="AM28" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN28" s="63" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO28" s="64" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP28" s="65" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ28" s="66" t="s">
+        <v>94</v>
+      </c>
+      <c r="AR28" s="65" t="s">
+        <v>94</v>
+      </c>
+      <c r="AS28" s="66" t="s">
+        <v>94</v>
+      </c>
+      <c r="AT28" s="66" t="s">
+        <v>94</v>
       </c>
       <c r="AU28" s="66" t="s">
         <v>94</v>
       </c>
       <c r="AV28" s="67" t="s">
-        <v>27</v>
-      </c>
-      <c r="AW28" s="65">
-        <v>0</v>
+        <v>94</v>
+      </c>
+      <c r="AW28" s="65" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:49" x14ac:dyDescent="0.25">
@@ -3601,7 +3604,7 @@
         <v>1</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>45</v>
@@ -3610,7 +3613,7 @@
         <v>1</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="6">
@@ -3671,7 +3674,7 @@
         <v>0.03</v>
       </c>
       <c r="AA29" s="32" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AB29" s="19">
         <v>3</v>
@@ -3694,43 +3697,43 @@
         <v>16933.333333333332</v>
       </c>
       <c r="AK29" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="AL29" s="58">
-        <v>1</v>
-      </c>
-      <c r="AM29" s="28">
-        <v>46508</v>
-      </c>
-      <c r="AN29" s="28">
-        <v>46873</v>
-      </c>
-      <c r="AO29" s="34">
-        <v>1.2380952380952381</v>
-      </c>
-      <c r="AP29" s="59">
-        <v>1300</v>
-      </c>
-      <c r="AQ29" s="60">
-        <v>15600</v>
-      </c>
-      <c r="AR29" s="59">
-        <v>25.7001647446458</v>
-      </c>
-      <c r="AS29" s="60">
-        <v>4.9359625940231758E-2</v>
-      </c>
-      <c r="AT29" s="60">
-        <v>1300</v>
-      </c>
-      <c r="AU29" s="60">
-        <v>250</v>
+        <v>94</v>
+      </c>
+      <c r="AL29" s="58" t="s">
+        <v>94</v>
+      </c>
+      <c r="AM29" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN29" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO29" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP29" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ29" s="60" t="s">
+        <v>94</v>
+      </c>
+      <c r="AR29" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="AS29" s="60" t="s">
+        <v>94</v>
+      </c>
+      <c r="AT29" s="60" t="s">
+        <v>94</v>
+      </c>
+      <c r="AU29" s="60" t="s">
+        <v>94</v>
       </c>
       <c r="AV29" s="61" t="s">
-        <v>27</v>
-      </c>
-      <c r="AW29" s="59">
-        <v>0</v>
+        <v>94</v>
+      </c>
+      <c r="AW29" s="59" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="30" spans="1:49" x14ac:dyDescent="0.25">
@@ -3741,16 +3744,16 @@
         <v>2</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E30" s="6">
         <v>2</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="6">
@@ -3811,7 +3814,7 @@
         <v>0.05</v>
       </c>
       <c r="AA30" s="32" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="AB30" s="19">
         <v>2</v>
@@ -3879,16 +3882,16 @@
         <v>3</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E31" s="6">
         <v>3</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G31" s="6"/>
       <c r="H31" s="6">
@@ -3949,7 +3952,7 @@
         <v>0</v>
       </c>
       <c r="AA31" s="32" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="AB31" s="19"/>
       <c r="AC31" s="19"/>
@@ -4024,7 +4027,7 @@
         <v>3</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G32" s="6"/>
       <c r="H32" s="6">
@@ -4229,7 +4232,7 @@
         <v>1</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>45</v>
@@ -4238,7 +4241,7 @@
         <v>1</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G34" s="6"/>
       <c r="H34" s="6">
@@ -4296,7 +4299,7 @@
         <v>46538</v>
       </c>
       <c r="Z34" s="52" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="AA34" s="32" t="s">
         <v>48</v>
@@ -4367,7 +4370,7 @@
         <v>2</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>45</v>
@@ -4376,7 +4379,7 @@
         <v>1</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G35" s="6"/>
       <c r="H35" s="6">
@@ -4434,7 +4437,7 @@
         <v>46706</v>
       </c>
       <c r="Z35" s="52" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="AA35" s="32" t="s">
         <v>48</v>
@@ -4505,7 +4508,7 @@
         <v>3</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>45</v>
@@ -4514,7 +4517,7 @@
         <v>1</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G36" s="6"/>
       <c r="H36" s="6">
@@ -4572,7 +4575,7 @@
         <v>47299</v>
       </c>
       <c r="Z36" s="52" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="AA36" s="32" t="s">
         <v>48</v>
@@ -4643,7 +4646,7 @@
         <v>4</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>45</v>
@@ -4652,7 +4655,7 @@
         <v>1</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="6">
@@ -4710,10 +4713,10 @@
         <v>47573</v>
       </c>
       <c r="Z37" s="52" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="AA37" s="32" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="AB37" s="19">
         <v>3</v>
@@ -4781,16 +4784,16 @@
         <v>5</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E38" s="6">
         <v>2</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G38" s="6"/>
       <c r="H38" s="6">
@@ -4848,10 +4851,10 @@
         <v>46996</v>
       </c>
       <c r="Z38" s="52" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="AA38" s="32" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AB38" s="19">
         <v>3</v>
@@ -4919,16 +4922,16 @@
         <v>6</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E39" s="6">
         <v>2</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G39" s="6"/>
       <c r="H39" s="6">
@@ -5059,16 +5062,16 @@
         <v>7</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E40" s="6">
         <v>2</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G40" s="6"/>
       <c r="H40" s="6">
@@ -5399,13 +5402,13 @@
     </row>
     <row r="45" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>53</v>
@@ -5414,7 +5417,7 @@
         <v>102</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>104</v>
@@ -5426,19 +5429,19 @@
         <v>106</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L45" s="1" t="s">
         <v>13</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N45" s="69" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="O45" s="69" t="s">
         <v>14</v>
@@ -5447,10 +5450,10 @@
         <v>26</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="R45" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="S45" s="1" t="s">
         <v>31</v>
@@ -5465,7 +5468,7 @@
         <v>37</v>
       </c>
       <c r="W45" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="AK45" s="22" t="s">
         <v>94</v>
@@ -5509,7 +5512,7 @@
     </row>
     <row r="46" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>8</v>
@@ -5518,10 +5521,10 @@
         <v>1</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F46" s="6">
         <v>0</v>
@@ -5617,7 +5620,7 @@
     </row>
     <row r="47" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>8</v>
@@ -5626,10 +5629,10 @@
         <v>1</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F47" s="6">
         <v>1</v>
@@ -5725,7 +5728,7 @@
     </row>
     <row r="48" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>8</v>
@@ -5734,10 +5737,10 @@
         <v>1</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F48" s="6">
         <v>2</v>
@@ -5833,7 +5836,7 @@
     </row>
     <row r="49" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>8</v>
@@ -5842,10 +5845,10 @@
         <v>1</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F49" s="6">
         <v>3</v>
@@ -5941,7 +5944,7 @@
     </row>
     <row r="50" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>8</v>
@@ -5950,10 +5953,10 @@
         <v>1</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F50" s="6">
         <v>4</v>
@@ -6049,7 +6052,7 @@
     </row>
     <row r="51" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>8</v>
@@ -6058,10 +6061,10 @@
         <v>1</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F51" s="6">
         <v>5</v>
@@ -6157,7 +6160,7 @@
     </row>
     <row r="52" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>8</v>
@@ -6166,10 +6169,10 @@
         <v>1</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F52" s="6">
         <v>6</v>
@@ -6226,7 +6229,7 @@
     </row>
     <row r="53" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B53" s="6" t="s">
         <v>8</v>
@@ -6235,10 +6238,10 @@
         <v>1</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F53" s="6">
         <v>7</v>
@@ -6293,7 +6296,7 @@
       </c>
       <c r="W53" s="13"/>
       <c r="AK53" s="72" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AL53" s="22"/>
       <c r="AM53" s="22"/>
@@ -6305,7 +6308,7 @@
     </row>
     <row r="54" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>8</v>
@@ -6314,10 +6317,10 @@
         <v>1</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F54" s="6">
         <v>8</v>
@@ -6372,33 +6375,33 @@
       </c>
       <c r="W54" s="13"/>
       <c r="AK54" s="56" t="s">
+        <v>151</v>
+      </c>
+      <c r="AL54" s="56" t="s">
         <v>152</v>
       </c>
-      <c r="AL54" s="56" t="s">
+      <c r="AM54" s="56" t="s">
         <v>153</v>
       </c>
-      <c r="AM54" s="56" t="s">
+      <c r="AN54" s="56" t="s">
         <v>154</v>
       </c>
-      <c r="AN54" s="56" t="s">
+      <c r="AO54" s="56" t="s">
         <v>155</v>
       </c>
-      <c r="AO54" s="56" t="s">
+      <c r="AP54" s="56" t="s">
         <v>156</v>
       </c>
-      <c r="AP54" s="56" t="s">
+      <c r="AQ54" s="56" t="s">
         <v>157</v>
       </c>
-      <c r="AQ54" s="56" t="s">
+      <c r="AR54" s="56" t="s">
         <v>158</v>
-      </c>
-      <c r="AR54" s="56" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="55" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>8</v>
@@ -6407,10 +6410,10 @@
         <v>1</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F55" s="6">
         <v>9</v>
@@ -6465,33 +6468,33 @@
       </c>
       <c r="W55" s="13"/>
       <c r="AK55" s="26" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="AL55" s="58">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AM55" s="28">
-        <v>45778</v>
+        <v>0</v>
       </c>
       <c r="AN55" s="28">
-        <v>46507</v>
-      </c>
-      <c r="AO55" s="59">
-        <v>958</v>
-      </c>
-      <c r="AP55" s="60">
-        <v>11496</v>
-      </c>
-      <c r="AQ55" s="59">
-        <v>1050</v>
-      </c>
-      <c r="AR55" s="60">
-        <v>12600</v>
+        <v>0</v>
+      </c>
+      <c r="AO55" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP55" s="60" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ55" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="AR55" s="60" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="56" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B56" s="6" t="s">
         <v>8</v>
@@ -6500,10 +6503,10 @@
         <v>1</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F56" s="6">
         <v>10</v>
@@ -6558,33 +6561,33 @@
       </c>
       <c r="W56" s="13"/>
       <c r="AK56" s="26" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AL56" s="58">
-        <v>1</v>
-      </c>
-      <c r="AM56" s="28">
-        <v>46508</v>
-      </c>
-      <c r="AN56" s="28">
-        <v>46873</v>
-      </c>
-      <c r="AO56" s="59">
-        <v>1300</v>
-      </c>
-      <c r="AP56" s="60">
-        <v>15600</v>
-      </c>
-      <c r="AQ56" s="59">
-        <v>1300</v>
-      </c>
-      <c r="AR56" s="60">
-        <v>15600</v>
+        <v>0</v>
+      </c>
+      <c r="AM56" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN56" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO56" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP56" s="60" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ56" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="AR56" s="60" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="57" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A57" s="73" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B57" s="73" t="s">
         <v>8</v>
@@ -6593,10 +6596,10 @@
         <v>1</v>
       </c>
       <c r="D57" s="73" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E57" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F57" s="73">
         <v>11</v>
@@ -6677,7 +6680,7 @@
     </row>
     <row r="58" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A58" s="73" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B58" s="73" t="s">
         <v>8</v>
@@ -6686,10 +6689,10 @@
         <v>1</v>
       </c>
       <c r="D58" s="73" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E58" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F58" s="73">
         <v>12</v>
@@ -6770,7 +6773,7 @@
     </row>
     <row r="59" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A59" s="73" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B59" s="73" t="s">
         <v>8</v>
@@ -6779,10 +6782,10 @@
         <v>1</v>
       </c>
       <c r="D59" s="73" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E59" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F59" s="73">
         <v>13</v>
@@ -6839,7 +6842,7 @@
     </row>
     <row r="60" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A60" s="73" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B60" s="73" t="s">
         <v>8</v>
@@ -6848,10 +6851,10 @@
         <v>1</v>
       </c>
       <c r="D60" s="73" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E60" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F60" s="73">
         <v>14</v>
@@ -6908,7 +6911,7 @@
     </row>
     <row r="61" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A61" s="73" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B61" s="73" t="s">
         <v>8</v>
@@ -6917,10 +6920,10 @@
         <v>1</v>
       </c>
       <c r="D61" s="73" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E61" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F61" s="73">
         <v>15</v>
@@ -6977,7 +6980,7 @@
     </row>
     <row r="62" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A62" s="78" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B62" s="78" t="s">
         <v>8</v>
@@ -6986,7 +6989,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="78" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E62" s="78" t="s">
         <v>163</v>
@@ -7046,7 +7049,7 @@
     </row>
     <row r="63" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A63" s="78" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B63" s="78" t="s">
         <v>8</v>
@@ -7055,7 +7058,7 @@
         <v>1</v>
       </c>
       <c r="D63" s="78" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E63" s="78" t="s">
         <v>163</v>
@@ -7115,7 +7118,7 @@
     </row>
     <row r="64" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A64" s="78" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B64" s="78" t="s">
         <v>8</v>
@@ -7124,7 +7127,7 @@
         <v>1</v>
       </c>
       <c r="D64" s="78" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E64" s="78" t="s">
         <v>163</v>
@@ -7184,7 +7187,7 @@
     </row>
     <row r="65" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A65" s="78" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B65" s="78" t="s">
         <v>8</v>
@@ -7193,7 +7196,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="78" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E65" s="78" t="s">
         <v>163</v>
@@ -7253,7 +7256,7 @@
     </row>
     <row r="66" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A66" s="78" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B66" s="78" t="s">
         <v>8</v>
@@ -7262,7 +7265,7 @@
         <v>1</v>
       </c>
       <c r="D66" s="78" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E66" s="78" t="s">
         <v>163</v>
@@ -7400,10 +7403,10 @@
         <v>2</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F68" s="6">
         <v>1</v>
@@ -7469,10 +7472,10 @@
         <v>2</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F69" s="6">
         <v>2</v>
@@ -7538,10 +7541,10 @@
         <v>2</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F70" s="6">
         <v>3</v>
@@ -7607,10 +7610,10 @@
         <v>2</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F71" s="6">
         <v>4</v>
@@ -7745,10 +7748,10 @@
         <v>3</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F73" s="6">
         <v>1</v>
@@ -7814,10 +7817,10 @@
         <v>3</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F74" s="6">
         <v>2</v>
@@ -7883,10 +7886,10 @@
         <v>3</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F75" s="6">
         <v>3</v>
@@ -7952,10 +7955,10 @@
         <v>3</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F76" s="6">
         <v>4</v>
@@ -8021,10 +8024,10 @@
         <v>3</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F77" s="6">
         <v>5</v>
@@ -8090,10 +8093,10 @@
         <v>3</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F78" s="6">
         <v>6</v>
@@ -8159,10 +8162,10 @@
         <v>3</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F79" s="6">
         <v>7</v>
@@ -8228,10 +8231,10 @@
         <v>3</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F80" s="6">
         <v>8</v>
@@ -8297,10 +8300,10 @@
         <v>3</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F81" s="6">
         <v>9</v>
@@ -8366,10 +8369,10 @@
         <v>3</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F82" s="6">
         <v>10</v>
@@ -8435,10 +8438,10 @@
         <v>3</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F83" s="6">
         <v>11</v>
@@ -8504,10 +8507,10 @@
         <v>3</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F84" s="6">
         <v>12</v>
@@ -8573,10 +8576,10 @@
         <v>3</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F85" s="6">
         <v>13</v>
@@ -8642,10 +8645,10 @@
         <v>3</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F86" s="6">
         <v>14</v>
@@ -8783,7 +8786,7 @@
         <v>112</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F88" s="6">
         <v>1</v>
@@ -8852,7 +8855,7 @@
         <v>112</v>
       </c>
       <c r="E89" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F89" s="6">
         <v>2</v>
@@ -8921,7 +8924,7 @@
         <v>112</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F90" s="6">
         <v>3</v>
@@ -8990,7 +8993,7 @@
         <v>112</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F91" s="6">
         <v>4</v>
@@ -9059,7 +9062,7 @@
         <v>112</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F92" s="6">
         <v>5</v>
@@ -9128,7 +9131,7 @@
         <v>112</v>
       </c>
       <c r="E93" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F93" s="6">
         <v>6</v>
@@ -9197,7 +9200,7 @@
         <v>112</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F94" s="6">
         <v>7</v>
@@ -9266,7 +9269,7 @@
         <v>112</v>
       </c>
       <c r="E95" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F95" s="6">
         <v>8</v>
@@ -9335,7 +9338,7 @@
         <v>112</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F96" s="6">
         <v>9</v>
@@ -9404,7 +9407,7 @@
         <v>112</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F97" s="6">
         <v>10</v>
@@ -9473,7 +9476,7 @@
         <v>112</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F98" s="6">
         <v>11</v>
@@ -9611,7 +9614,7 @@
         <v>95</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F100" s="6">
         <v>1</v>
@@ -9680,7 +9683,7 @@
         <v>95</v>
       </c>
       <c r="E101" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F101" s="6">
         <v>2</v>
@@ -9749,7 +9752,7 @@
         <v>95</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F102" s="6">
         <v>3</v>
@@ -9818,7 +9821,7 @@
         <v>95</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F103" s="6">
         <v>4</v>
@@ -9887,7 +9890,7 @@
         <v>95</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F104" s="6">
         <v>5</v>
@@ -9956,7 +9959,7 @@
         <v>95</v>
       </c>
       <c r="E105" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F105" s="6">
         <v>6</v>
@@ -10025,7 +10028,7 @@
         <v>95</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F106" s="6">
         <v>7</v>
@@ -10094,7 +10097,7 @@
         <v>95</v>
       </c>
       <c r="E107" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F107" s="6">
         <v>8</v>
@@ -10163,7 +10166,7 @@
         <v>95</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F108" s="6">
         <v>9</v>
@@ -10232,7 +10235,7 @@
         <v>95</v>
       </c>
       <c r="E109" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F109" s="6">
         <v>10</v>
@@ -10301,7 +10304,7 @@
         <v>95</v>
       </c>
       <c r="E110" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F110" s="73">
         <v>11</v>
@@ -10370,7 +10373,7 @@
         <v>95</v>
       </c>
       <c r="E111" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F111" s="73">
         <v>12</v>
@@ -10439,7 +10442,7 @@
         <v>95</v>
       </c>
       <c r="E112" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F112" s="73">
         <v>13</v>
@@ -10508,7 +10511,7 @@
         <v>95</v>
       </c>
       <c r="E113" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F113" s="73">
         <v>14</v>
@@ -10577,7 +10580,7 @@
         <v>95</v>
       </c>
       <c r="E114" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F114" s="73">
         <v>15</v>
@@ -10715,7 +10718,7 @@
         <v>100</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F116" s="6">
         <v>1</v>
@@ -10784,7 +10787,7 @@
         <v>100</v>
       </c>
       <c r="E117" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F117" s="6">
         <v>2</v>
@@ -10853,7 +10856,7 @@
         <v>100</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F118" s="6">
         <v>3</v>
@@ -10922,7 +10925,7 @@
         <v>100</v>
       </c>
       <c r="E119" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F119" s="6">
         <v>4</v>
@@ -10991,7 +10994,7 @@
         <v>100</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F120" s="6">
         <v>5</v>
@@ -11060,7 +11063,7 @@
         <v>100</v>
       </c>
       <c r="E121" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F121" s="73">
         <v>6</v>
@@ -11129,7 +11132,7 @@
         <v>100</v>
       </c>
       <c r="E122" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F122" s="73">
         <v>7</v>
@@ -11198,7 +11201,7 @@
         <v>100</v>
       </c>
       <c r="E123" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F123" s="73">
         <v>8</v>
@@ -11267,7 +11270,7 @@
         <v>100</v>
       </c>
       <c r="E124" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F124" s="73">
         <v>9</v>
@@ -11336,7 +11339,7 @@
         <v>100</v>
       </c>
       <c r="E125" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F125" s="73">
         <v>10</v>
@@ -11474,7 +11477,7 @@
         <v>112</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F127" s="6">
         <v>1</v>
@@ -11543,7 +11546,7 @@
         <v>112</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F128" s="6">
         <v>2</v>
@@ -11612,7 +11615,7 @@
         <v>112</v>
       </c>
       <c r="E129" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F129" s="6">
         <v>3</v>
@@ -11681,7 +11684,7 @@
         <v>112</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F130" s="6">
         <v>4</v>
@@ -11750,7 +11753,7 @@
         <v>112</v>
       </c>
       <c r="E131" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F131" s="6">
         <v>5</v>
@@ -11819,7 +11822,7 @@
         <v>112</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F132" s="6">
         <v>6</v>
@@ -11888,7 +11891,7 @@
         <v>112</v>
       </c>
       <c r="E133" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F133" s="6">
         <v>7</v>
@@ -11957,7 +11960,7 @@
         <v>112</v>
       </c>
       <c r="E134" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F134" s="6">
         <v>8</v>
@@ -12026,7 +12029,7 @@
         <v>112</v>
       </c>
       <c r="E135" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F135" s="6">
         <v>9</v>
@@ -12095,7 +12098,7 @@
         <v>112</v>
       </c>
       <c r="E136" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F136" s="6">
         <v>10</v>
@@ -12164,7 +12167,7 @@
         <v>112</v>
       </c>
       <c r="E137" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F137" s="6">
         <v>11</v>
@@ -12299,10 +12302,10 @@
         <v>1</v>
       </c>
       <c r="D139" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E139" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F139" s="6">
         <v>1</v>
@@ -12368,10 +12371,10 @@
         <v>1</v>
       </c>
       <c r="D140" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E140" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F140" s="6">
         <v>2</v>
@@ -12437,10 +12440,10 @@
         <v>1</v>
       </c>
       <c r="D141" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E141" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F141" s="6">
         <v>3</v>
@@ -12506,10 +12509,10 @@
         <v>1</v>
       </c>
       <c r="D142" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F142" s="6">
         <v>4</v>
@@ -12575,10 +12578,10 @@
         <v>1</v>
       </c>
       <c r="D143" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E143" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F143" s="6">
         <v>5</v>
@@ -12713,10 +12716,10 @@
         <v>2</v>
       </c>
       <c r="D145" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E145" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F145" s="6">
         <v>1</v>
@@ -12782,10 +12785,10 @@
         <v>2</v>
       </c>
       <c r="D146" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E146" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F146" s="6">
         <v>2</v>
@@ -12851,10 +12854,10 @@
         <v>2</v>
       </c>
       <c r="D147" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E147" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F147" s="6">
         <v>3</v>
@@ -12920,10 +12923,10 @@
         <v>2</v>
       </c>
       <c r="D148" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E148" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F148" s="6">
         <v>4</v>
@@ -12989,10 +12992,10 @@
         <v>2</v>
       </c>
       <c r="D149" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E149" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F149" s="6">
         <v>5</v>
@@ -13125,10 +13128,10 @@
         <v>3</v>
       </c>
       <c r="D151" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E151" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F151" s="6">
         <v>1</v>
@@ -13194,10 +13197,10 @@
         <v>3</v>
       </c>
       <c r="D152" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E152" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F152" s="6">
         <v>2</v>
@@ -13263,10 +13266,10 @@
         <v>3</v>
       </c>
       <c r="D153" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E153" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F153" s="6">
         <v>3</v>
@@ -13332,10 +13335,10 @@
         <v>3</v>
       </c>
       <c r="D154" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E154" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F154" s="6">
         <v>4</v>
@@ -13401,10 +13404,10 @@
         <v>3</v>
       </c>
       <c r="D155" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E155" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F155" s="6">
         <v>5</v>
@@ -13539,10 +13542,10 @@
         <v>4</v>
       </c>
       <c r="D157" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E157" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F157" s="6">
         <v>1</v>
@@ -13608,10 +13611,10 @@
         <v>4</v>
       </c>
       <c r="D158" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E158" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F158" s="6">
         <v>2</v>
@@ -13677,10 +13680,10 @@
         <v>4</v>
       </c>
       <c r="D159" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E159" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F159" s="6">
         <v>3</v>
@@ -13746,10 +13749,10 @@
         <v>4</v>
       </c>
       <c r="D160" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E160" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F160" s="6">
         <v>4</v>
@@ -13815,10 +13818,10 @@
         <v>4</v>
       </c>
       <c r="D161" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E161" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F161" s="6">
         <v>5</v>
@@ -13884,10 +13887,10 @@
         <v>4</v>
       </c>
       <c r="D162" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E162" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F162" s="6">
         <v>6</v>
@@ -13953,10 +13956,10 @@
         <v>4</v>
       </c>
       <c r="D163" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E163" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F163" s="6">
         <v>7</v>
@@ -14022,10 +14025,10 @@
         <v>4</v>
       </c>
       <c r="D164" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E164" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F164" s="6">
         <v>8</v>
@@ -14091,10 +14094,10 @@
         <v>4</v>
       </c>
       <c r="D165" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E165" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F165" s="6">
         <v>9</v>
@@ -14160,10 +14163,10 @@
         <v>4</v>
       </c>
       <c r="D166" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E166" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F166" s="6">
         <v>10</v>
@@ -14229,10 +14232,10 @@
         <v>4</v>
       </c>
       <c r="D167" s="73" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E167" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F167" s="73">
         <v>11</v>
@@ -14298,10 +14301,10 @@
         <v>4</v>
       </c>
       <c r="D168" s="73" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E168" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F168" s="73">
         <v>12</v>
@@ -14367,10 +14370,10 @@
         <v>4</v>
       </c>
       <c r="D169" s="73" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E169" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F169" s="73">
         <v>13</v>
@@ -14436,10 +14439,10 @@
         <v>4</v>
       </c>
       <c r="D170" s="73" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E170" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F170" s="73">
         <v>14</v>
@@ -14505,10 +14508,10 @@
         <v>4</v>
       </c>
       <c r="D171" s="73" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E171" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F171" s="73">
         <v>15</v>
@@ -14574,7 +14577,7 @@
         <v>4</v>
       </c>
       <c r="D172" s="78" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E172" s="78" t="s">
         <v>163</v>
@@ -14643,7 +14646,7 @@
         <v>4</v>
       </c>
       <c r="D173" s="78" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E173" s="78" t="s">
         <v>163</v>
@@ -14712,7 +14715,7 @@
         <v>4</v>
       </c>
       <c r="D174" s="78" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E174" s="78" t="s">
         <v>163</v>
@@ -14781,7 +14784,7 @@
         <v>4</v>
       </c>
       <c r="D175" s="78" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E175" s="78" t="s">
         <v>163</v>
@@ -14850,7 +14853,7 @@
         <v>4</v>
       </c>
       <c r="D176" s="78" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E176" s="78" t="s">
         <v>163</v>
@@ -14919,7 +14922,7 @@
         <v>4</v>
       </c>
       <c r="D177" s="86" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E177" s="86" t="s">
         <v>175</v>
@@ -14988,7 +14991,7 @@
         <v>4</v>
       </c>
       <c r="D178" s="86" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E178" s="86" t="s">
         <v>175</v>
@@ -15057,7 +15060,7 @@
         <v>4</v>
       </c>
       <c r="D179" s="86" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E179" s="86" t="s">
         <v>175</v>
@@ -15126,7 +15129,7 @@
         <v>4</v>
       </c>
       <c r="D180" s="86" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E180" s="86" t="s">
         <v>175</v>
@@ -15195,7 +15198,7 @@
         <v>4</v>
       </c>
       <c r="D181" s="86" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E181" s="86" t="s">
         <v>175</v>
@@ -15333,10 +15336,10 @@
         <v>5</v>
       </c>
       <c r="D183" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E183" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F183" s="6">
         <v>1</v>
@@ -15402,10 +15405,10 @@
         <v>5</v>
       </c>
       <c r="D184" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E184" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F184" s="6">
         <v>2</v>
@@ -15471,10 +15474,10 @@
         <v>5</v>
       </c>
       <c r="D185" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E185" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F185" s="6">
         <v>3</v>
@@ -15540,10 +15543,10 @@
         <v>5</v>
       </c>
       <c r="D186" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E186" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F186" s="6">
         <v>4</v>
@@ -15609,10 +15612,10 @@
         <v>5</v>
       </c>
       <c r="D187" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E187" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F187" s="6">
         <v>5</v>
@@ -15678,10 +15681,10 @@
         <v>5</v>
       </c>
       <c r="D188" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E188" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F188" s="6">
         <v>6</v>
@@ -15747,7 +15750,7 @@
         <v>5</v>
       </c>
       <c r="D189" s="78" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E189" s="78" t="s">
         <v>163</v>
@@ -15816,7 +15819,7 @@
         <v>5</v>
       </c>
       <c r="D190" s="78" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E190" s="78" t="s">
         <v>163</v>
@@ -15954,10 +15957,10 @@
         <v>6</v>
       </c>
       <c r="D192" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E192" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F192" s="6">
         <v>1</v>
@@ -16092,10 +16095,10 @@
         <v>7</v>
       </c>
       <c r="D194" s="6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E194" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F194" s="6">
         <v>1</v>
@@ -16227,13 +16230,13 @@
         <v>6</v>
       </c>
       <c r="C196" s="6">
-        <v>1</v>
+        <v>102</v>
       </c>
       <c r="D196" s="6" t="s">
         <v>44</v>
       </c>
       <c r="E196" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F196" s="6">
         <v>1</v>
@@ -16365,13 +16368,13 @@
         <v>6</v>
       </c>
       <c r="C198" s="6">
-        <v>2</v>
+        <v>104</v>
       </c>
       <c r="D198" s="6" t="s">
         <v>51</v>
       </c>
       <c r="E198" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F198" s="6">
         <v>1</v>
@@ -16434,13 +16437,13 @@
         <v>6</v>
       </c>
       <c r="C199" s="6">
-        <v>2</v>
+        <v>104</v>
       </c>
       <c r="D199" s="6" t="s">
         <v>51</v>
       </c>
       <c r="E199" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F199" s="6">
         <v>1</v>
@@ -16572,13 +16575,13 @@
         <v>6</v>
       </c>
       <c r="C201" s="6">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D201" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E201" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F201" s="6">
         <v>1</v>
@@ -16641,13 +16644,13 @@
         <v>6</v>
       </c>
       <c r="C202" s="6">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D202" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E202" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F202" s="6">
         <v>2</v>
@@ -16710,13 +16713,13 @@
         <v>6</v>
       </c>
       <c r="C203" s="6">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D203" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E203" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F203" s="6">
         <v>3</v>
@@ -16779,13 +16782,13 @@
         <v>6</v>
       </c>
       <c r="C204" s="6">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D204" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E204" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F204" s="6">
         <v>4</v>
@@ -16848,13 +16851,13 @@
         <v>6</v>
       </c>
       <c r="C205" s="6">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D205" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E205" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F205" s="6">
         <v>5</v>
@@ -16917,13 +16920,13 @@
         <v>6</v>
       </c>
       <c r="C206" s="6">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D206" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E206" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F206" s="6">
         <v>6</v>
@@ -16986,13 +16989,13 @@
         <v>6</v>
       </c>
       <c r="C207" s="73">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D207" s="73" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E207" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F207" s="73">
         <v>7</v>
@@ -17055,13 +17058,13 @@
         <v>6</v>
       </c>
       <c r="C208" s="73">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D208" s="73" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E208" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F208" s="73">
         <v>8</v>
@@ -17124,13 +17127,13 @@
         <v>6</v>
       </c>
       <c r="C209" s="73">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D209" s="73" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E209" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F209" s="73">
         <v>9</v>
@@ -17193,13 +17196,13 @@
         <v>6</v>
       </c>
       <c r="C210" s="73">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D210" s="73" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E210" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F210" s="73">
         <v>10</v>
@@ -17262,13 +17265,13 @@
         <v>6</v>
       </c>
       <c r="C211" s="73">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D211" s="73" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E211" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F211" s="73">
         <v>11</v>
@@ -17331,10 +17334,10 @@
         <v>6</v>
       </c>
       <c r="C212" s="78">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D212" s="78" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E212" s="78" t="s">
         <v>163</v>
@@ -17400,10 +17403,10 @@
         <v>6</v>
       </c>
       <c r="C213" s="78">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D213" s="78" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E213" s="78" t="s">
         <v>163</v>
@@ -17469,10 +17472,10 @@
         <v>6</v>
       </c>
       <c r="C214" s="78">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D214" s="78" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E214" s="78" t="s">
         <v>163</v>
@@ -17538,10 +17541,10 @@
         <v>6</v>
       </c>
       <c r="C215" s="78">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D215" s="78" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E215" s="78" t="s">
         <v>163</v>
@@ -17607,10 +17610,10 @@
         <v>6</v>
       </c>
       <c r="C216" s="78">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="D216" s="78" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E216" s="78" t="s">
         <v>163</v>
@@ -17745,13 +17748,13 @@
         <v>6</v>
       </c>
       <c r="C218" s="6">
-        <v>4</v>
+        <v>108</v>
       </c>
       <c r="D218" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E218" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F218" s="6">
         <v>1</v>
@@ -17814,13 +17817,13 @@
         <v>6</v>
       </c>
       <c r="C219" s="6">
-        <v>4</v>
+        <v>108</v>
       </c>
       <c r="D219" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E219" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F219" s="6">
         <v>2</v>
@@ -17883,13 +17886,13 @@
         <v>6</v>
       </c>
       <c r="C220" s="6">
-        <v>4</v>
+        <v>108</v>
       </c>
       <c r="D220" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E220" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F220" s="6">
         <v>3</v>
@@ -17952,13 +17955,13 @@
         <v>6</v>
       </c>
       <c r="C221" s="6">
-        <v>4</v>
+        <v>108</v>
       </c>
       <c r="D221" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E221" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F221" s="6">
         <v>4</v>
@@ -18021,13 +18024,13 @@
         <v>6</v>
       </c>
       <c r="C222" s="6">
-        <v>4</v>
+        <v>108</v>
       </c>
       <c r="D222" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E222" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F222" s="6">
         <v>5</v>
@@ -18090,13 +18093,13 @@
         <v>6</v>
       </c>
       <c r="C223" s="6">
-        <v>4</v>
+        <v>108</v>
       </c>
       <c r="D223" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E223" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F223" s="6">
         <v>6</v>
@@ -18231,10 +18234,10 @@
         <v>201</v>
       </c>
       <c r="D225" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E225" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F225" s="6">
         <v>1</v>
@@ -18360,7 +18363,7 @@
     </row>
     <row r="227" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A227" s="6" t="s">
-        <v>50</v>
+        <v>184</v>
       </c>
       <c r="B227" s="6" t="s">
         <v>6</v>
@@ -18369,10 +18372,10 @@
         <v>202</v>
       </c>
       <c r="D227" s="6" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E227" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F227" s="6">
         <v>1</v>
@@ -18429,7 +18432,7 @@
     </row>
     <row r="228" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A228" s="6" t="s">
-        <v>50</v>
+        <v>184</v>
       </c>
       <c r="B228" s="6" t="s">
         <v>6</v>
@@ -18438,10 +18441,10 @@
         <v>202</v>
       </c>
       <c r="D228" s="6" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E228" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F228" s="6">
         <v>1</v>
@@ -18498,7 +18501,7 @@
     </row>
     <row r="229" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A229" s="73" t="s">
-        <v>50</v>
+        <v>184</v>
       </c>
       <c r="B229" s="73" t="s">
         <v>6</v>
@@ -18507,10 +18510,10 @@
         <v>202</v>
       </c>
       <c r="D229" s="73" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E229" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F229" s="73">
         <v>1</v>
@@ -18636,7 +18639,7 @@
     </row>
     <row r="231" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A231" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B231" s="6" t="s">
         <v>6</v>
@@ -18648,7 +18651,7 @@
         <v>71</v>
       </c>
       <c r="E231" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F231" s="6">
         <v>1</v>
@@ -18705,7 +18708,7 @@
     </row>
     <row r="232" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A232" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B232" s="6" t="s">
         <v>6</v>
@@ -18717,7 +18720,7 @@
         <v>71</v>
       </c>
       <c r="E232" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F232" s="6">
         <v>2</v>
@@ -18774,7 +18777,7 @@
     </row>
     <row r="233" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A233" s="73" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B233" s="73" t="s">
         <v>6</v>
@@ -18786,7 +18789,7 @@
         <v>71</v>
       </c>
       <c r="E233" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F233" s="73">
         <v>3</v>
@@ -18843,7 +18846,7 @@
     </row>
     <row r="234" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A234" s="78" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B234" s="78" t="s">
         <v>6</v>
@@ -18981,7 +18984,7 @@
     </row>
     <row r="236" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A236" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B236" s="6" t="s">
         <v>6</v>
@@ -18993,7 +18996,7 @@
         <v>75</v>
       </c>
       <c r="E236" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F236" s="6">
         <v>1</v>
@@ -19119,7 +19122,7 @@
     </row>
     <row r="238" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A238" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B238" s="6" t="s">
         <v>6</v>
@@ -19131,7 +19134,7 @@
         <v>78</v>
       </c>
       <c r="E238" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F238" s="6">
         <v>1</v>
@@ -19188,7 +19191,7 @@
     </row>
     <row r="239" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A239" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B239" s="6" t="s">
         <v>6</v>
@@ -19200,7 +19203,7 @@
         <v>78</v>
       </c>
       <c r="E239" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F239" s="6">
         <v>2</v>
@@ -19257,7 +19260,7 @@
     </row>
     <row r="240" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A240" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B240" s="6" t="s">
         <v>6</v>
@@ -19269,7 +19272,7 @@
         <v>78</v>
       </c>
       <c r="E240" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F240" s="6">
         <v>3</v>
@@ -19395,7 +19398,7 @@
     </row>
     <row r="242" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A242" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B242" s="6" t="s">
         <v>6</v>
@@ -19407,7 +19410,7 @@
         <v>91</v>
       </c>
       <c r="E242" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F242" s="6">
         <v>1</v>
@@ -19464,7 +19467,7 @@
     </row>
     <row r="243" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A243" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B243" s="6" t="s">
         <v>6</v>
@@ -19476,7 +19479,7 @@
         <v>91</v>
       </c>
       <c r="E243" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F243" s="6">
         <v>2</v>
@@ -19533,7 +19536,7 @@
     </row>
     <row r="244" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A244" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B244" s="6" t="s">
         <v>6</v>
@@ -19545,7 +19548,7 @@
         <v>91</v>
       </c>
       <c r="E244" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F244" s="6">
         <v>3</v>
@@ -19671,7 +19674,7 @@
     </row>
     <row r="246" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A246" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B246" s="6" t="s">
         <v>6</v>
@@ -19683,7 +19686,7 @@
         <v>80</v>
       </c>
       <c r="E246" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F246" s="6">
         <v>1</v>
@@ -19740,7 +19743,7 @@
     </row>
     <row r="247" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A247" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B247" s="6" t="s">
         <v>6</v>
@@ -19752,7 +19755,7 @@
         <v>80</v>
       </c>
       <c r="E247" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F247" s="6">
         <v>1</v>
@@ -19811,7 +19814,7 @@
     </row>
     <row r="248" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A248" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B248" s="6" t="s">
         <v>6</v>
@@ -19823,7 +19826,7 @@
         <v>80</v>
       </c>
       <c r="E248" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F248" s="6">
         <v>1</v>
@@ -19882,7 +19885,7 @@
     </row>
     <row r="249" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A249" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B249" s="6" t="s">
         <v>6</v>
@@ -19894,7 +19897,7 @@
         <v>80</v>
       </c>
       <c r="E249" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F249" s="6">
         <v>1</v>
@@ -19953,7 +19956,7 @@
     </row>
     <row r="250" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A250" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B250" s="6" t="s">
         <v>6</v>
@@ -19965,7 +19968,7 @@
         <v>80</v>
       </c>
       <c r="E250" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F250" s="6">
         <v>1</v>
@@ -20024,7 +20027,7 @@
     </row>
     <row r="251" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A251" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B251" s="6" t="s">
         <v>6</v>
@@ -20036,7 +20039,7 @@
         <v>80</v>
       </c>
       <c r="E251" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F251" s="6">
         <v>1</v>
@@ -20164,7 +20167,7 @@
     </row>
     <row r="253" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A253" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B253" s="6" t="s">
         <v>6</v>
@@ -20176,7 +20179,7 @@
         <v>85</v>
       </c>
       <c r="E253" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F253" s="6">
         <v>1</v>
@@ -20233,7 +20236,7 @@
     </row>
     <row r="254" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A254" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B254" s="6" t="s">
         <v>6</v>
@@ -20245,7 +20248,7 @@
         <v>85</v>
       </c>
       <c r="E254" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F254" s="6">
         <v>2</v>
@@ -20302,7 +20305,7 @@
     </row>
     <row r="255" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A255" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B255" s="6" t="s">
         <v>6</v>
@@ -20314,7 +20317,7 @@
         <v>85</v>
       </c>
       <c r="E255" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F255" s="6">
         <v>3</v>
@@ -20371,7 +20374,7 @@
     </row>
     <row r="256" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A256" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B256" s="6" t="s">
         <v>6</v>
@@ -20383,7 +20386,7 @@
         <v>85</v>
       </c>
       <c r="E256" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F256" s="6">
         <v>4</v>
@@ -20440,7 +20443,7 @@
     </row>
     <row r="257" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A257" s="73" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B257" s="73" t="s">
         <v>6</v>
@@ -20452,7 +20455,7 @@
         <v>85</v>
       </c>
       <c r="E257" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F257" s="73">
         <v>5</v>
@@ -20509,7 +20512,7 @@
     </row>
     <row r="258" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A258" s="73" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B258" s="73" t="s">
         <v>6</v>
@@ -20521,7 +20524,7 @@
         <v>85</v>
       </c>
       <c r="E258" s="73" t="s">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="F258" s="73">
         <v>6</v>
@@ -20647,7 +20650,7 @@
     </row>
     <row r="260" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A260" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B260" s="6" t="s">
         <v>6</v>
@@ -20659,7 +20662,7 @@
         <v>90</v>
       </c>
       <c r="E260" s="6" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="F260" s="6">
         <v>1</v>

</xml_diff>

<commit_message>
Dashboard update Tue 05/12/2026 21:17
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B7B0ED2-E838-467F-9B77-D5FDDB1D1043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{65D6DE4E-3BD6-425B-8FBE-57F760437E1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4890" yWindow="2505" windowWidth="52710" windowHeight="29895" xr2:uid="{3EBA7C37-EF48-42B6-AFC8-6B42723A749E}"/>
+    <workbookView xWindow="3900" yWindow="2505" windowWidth="52710" windowHeight="29895" xr2:uid="{D1DE1A64-D3AF-4AC7-A8E4-251A3C5B9995}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1358,7 +1358,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39BF2352-2549-4FEC-ACAC-8E7C8FEE077F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A91FA5B-2706-42F8-B8A4-697676A78052}">
   <dimension ref="A1:AW260"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2404,7 +2404,7 @@
         <v>74</v>
       </c>
       <c r="AN17" s="31">
-        <v>46348.599200000004</v>
+        <v>43688</v>
       </c>
       <c r="AS17" s="23" t="s">
         <v>75</v>
@@ -3870,7 +3870,7 @@
         <v>0.6</v>
       </c>
       <c r="AT30" s="66">
-        <v>46348.599200000004</v>
+        <v>43688</v>
       </c>
       <c r="AU30" s="66" t="s">
         <v>96</v>
@@ -4009,7 +4009,7 @@
         <v>47739.057176000002</v>
       </c>
       <c r="AU31" s="60">
-        <v>1390.4579759999979</v>
+        <v>4051.0571760000021</v>
       </c>
       <c r="AV31" s="61" t="s">
         <v>47</v>
@@ -5679,7 +5679,7 @@
         <v>21.500004921259844</v>
       </c>
       <c r="R47" s="13">
-        <v>43688.01</v>
+        <v>43688</v>
       </c>
       <c r="S47" s="70">
         <v>45383</v>
@@ -5787,7 +5787,7 @@
         <v>44.29</v>
       </c>
       <c r="R48" s="71">
-        <v>43688.01</v>
+        <v>43688</v>
       </c>
       <c r="S48" s="16">
         <v>45383</v>
@@ -5894,8 +5894,8 @@
       <c r="Q49" s="13">
         <v>45.618700000000004</v>
       </c>
-      <c r="R49" s="13">
-        <v>46348.599200000004</v>
+      <c r="R49" s="71">
+        <v>43688</v>
       </c>
       <c r="S49" s="16">
         <v>45383</v>

</xml_diff>

<commit_message>
Dashboard update Tue 05/12/2026 22:08
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AD47716-537A-4A22-BB21-1E2F6F378D7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{458BC4D3-B259-4146-BE7D-C6565AD9B8C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="390" windowWidth="76740" windowHeight="29895" xr2:uid="{75AC79F8-51D6-451A-BA5E-F59182317FA2}"/>
+    <workbookView xWindow="0" yWindow="1170" windowWidth="76740" windowHeight="29895" xr2:uid="{ABD13070-944B-4C96-89F5-E5D4D5548C69}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1364,7 +1364,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB15EA63-138B-483C-BECA-67C4905E8192}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31E38054-2EAC-4B8A-97D1-C6E85A881457}">
   <dimension ref="A1:AW260"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -13258,7 +13258,7 @@
         <v>32.250489236790607</v>
       </c>
       <c r="R152" s="75">
-        <v>8300</v>
+        <v>8299.9500000000007</v>
       </c>
       <c r="S152" s="17">
         <v>43631</v>

</xml_diff>

<commit_message>
Dashboard update Wed 05/13/2026  6:36
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{458BC4D3-B259-4146-BE7D-C6565AD9B8C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{60B5315B-A78F-4A95-9323-D9515CD2AC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1170" windowWidth="76740" windowHeight="29895" xr2:uid="{ABD13070-944B-4C96-89F5-E5D4D5548C69}"/>
+    <workbookView xWindow="0" yWindow="2505" windowWidth="76740" windowHeight="29895" xr2:uid="{7836C6DC-3EDD-4328-AF62-4D3841D4D0AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -473,7 +473,7 @@
     <t>203_Apt</t>
   </si>
   <si>
-    <t>Alan DiEsso</t>
+    <t>Gary DiEsso</t>
   </si>
   <si>
     <t>ID</t>
@@ -581,7 +581,7 @@
     <t>1280 Springfield_202_Apt_VACANT_6</t>
   </si>
   <si>
-    <t>1280 Springfield_203_Apt_Alan DiEsso</t>
+    <t>1280 Springfield_203_Apt_Gary DiEsso</t>
   </si>
   <si>
     <t>114 Central_102_Nabig Sakr</t>
@@ -1364,7 +1364,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31E38054-2EAC-4B8A-97D1-C6E85A881457}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{184512F1-06E0-462E-BFCD-6356E62C4150}">
   <dimension ref="A1:AW260"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2184,7 +2184,7 @@
         <v>66</v>
       </c>
       <c r="AT15" s="32">
-        <v>28.066666666666666</v>
+        <v>28.033333333333335</v>
       </c>
     </row>
     <row r="16" spans="1:48" x14ac:dyDescent="0.25">
@@ -2485,13 +2485,13 @@
         <v>-10.571254319983737</v>
       </c>
       <c r="W18" s="17">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="X18" s="17">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="Y18" s="17">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="Z18" s="18"/>
       <c r="AA18" s="19" t="s">
@@ -2989,13 +2989,13 @@
         <v>66</v>
       </c>
       <c r="AN22" s="32">
-        <v>28.066666666666666</v>
+        <v>28.033333333333335</v>
       </c>
       <c r="AS22" s="25" t="s">
         <v>66</v>
       </c>
       <c r="AT22" s="41">
-        <v>4.9000000000000004</v>
+        <v>4.8666666666666663</v>
       </c>
     </row>
     <row r="23" spans="1:49" x14ac:dyDescent="0.25">
@@ -13258,7 +13258,7 @@
         <v>32.250489236790607</v>
       </c>
       <c r="R152" s="75">
-        <v>8299.9500000000007</v>
+        <v>8300</v>
       </c>
       <c r="S152" s="17">
         <v>43631</v>
@@ -19021,10 +19021,10 @@
         <v>1</v>
       </c>
       <c r="G236" s="97">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="H236" s="97">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="I236" s="11">
         <v>0</v>
@@ -19057,13 +19057,13 @@
         <v>0</v>
       </c>
       <c r="S236" s="74">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="T236" s="74">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="U236" s="74">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="V236" s="14">
         <v>0</v>

</xml_diff>

<commit_message>
Dashboard update Wed 05/13/2026  6:40
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{60B5315B-A78F-4A95-9323-D9515CD2AC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{54109B08-E85C-4C40-AC19-E2ABA2965B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2505" windowWidth="76740" windowHeight="29895" xr2:uid="{7836C6DC-3EDD-4328-AF62-4D3841D4D0AC}"/>
+    <workbookView xWindow="0" yWindow="2505" windowWidth="76740" windowHeight="29895" xr2:uid="{AA865F56-9907-4CCB-98DA-821957C2BF23}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1364,7 +1364,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{184512F1-06E0-462E-BFCD-6356E62C4150}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAD7EC12-EF6E-4A06-AA24-D161A1B68BBA}">
   <dimension ref="A1:AW260"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -13258,7 +13258,7 @@
         <v>32.250489236790607</v>
       </c>
       <c r="R152" s="75">
-        <v>8300</v>
+        <v>8299.9500000000007</v>
       </c>
       <c r="S152" s="17">
         <v>43631</v>

</xml_diff>

<commit_message>
Dashboard update Sat 05/16/2026  6:22
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{26711B88-8415-4F79-8D24-5286C2BB357F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C35D5FE7-5C03-4483-A71C-F4A8F6442E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1200" yWindow="2505" windowWidth="56400" windowHeight="29895" xr2:uid="{7A321B7E-018A-4423-AAE2-A9BCD4FB6406}"/>
+    <workbookView xWindow="1200" yWindow="2505" windowWidth="56400" windowHeight="29895" xr2:uid="{315CDE70-047F-4E1E-9E2C-A2F9F7222378}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -628,7 +628,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -696,7 +696,6 @@
     <xf numFmtId="44" fontId="2" fillId="9" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
@@ -1034,7 +1033,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A85AC4B-68A9-41CE-9691-6468B00C91F2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6B787EC-957D-4A2C-9B3C-BF22C0723396}">
   <dimension ref="A1:AI261"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -4324,7 +4323,7 @@
       <c r="F47" s="6">
         <v>1</v>
       </c>
-      <c r="G47" s="15">
+      <c r="G47" s="36">
         <v>45566</v>
       </c>
       <c r="H47" s="36">
@@ -5846,7 +5845,7 @@
         <v>0.05</v>
       </c>
       <c r="J68" s="12">
-        <v>8775</v>
+        <v>8755</v>
       </c>
       <c r="K68" s="12">
         <v>105300</v>
@@ -5870,7 +5869,7 @@
         <v>25.077399380804952</v>
       </c>
       <c r="R68" s="12">
-        <v>17550</v>
+        <v>17510</v>
       </c>
       <c r="S68" s="36">
         <v>38504</v>
@@ -5879,7 +5878,7 @@
         <v>38504</v>
       </c>
       <c r="U68" s="36">
-        <v>47543</v>
+        <v>47542</v>
       </c>
       <c r="V68" s="12">
         <v>0</v>
@@ -5915,7 +5914,7 @@
         <v>46446</v>
       </c>
       <c r="I69" s="9">
-        <v>5.4131054131054235E-2</v>
+        <v>5.6539120502570039E-2</v>
       </c>
       <c r="J69" s="12">
         <v>9250</v>
@@ -5951,7 +5950,7 @@
         <v>38504</v>
       </c>
       <c r="U69" s="15">
-        <v>47543</v>
+        <v>47542</v>
       </c>
       <c r="V69" s="12">
         <v>0</v>
@@ -6023,7 +6022,7 @@
         <v>38504</v>
       </c>
       <c r="U70" s="15">
-        <v>47543</v>
+        <v>47542</v>
       </c>
       <c r="V70" s="12">
         <v>0</v>
@@ -6056,7 +6055,7 @@
         <v>46813</v>
       </c>
       <c r="H71" s="15">
-        <v>47178</v>
+        <v>47177</v>
       </c>
       <c r="I71" s="9">
         <v>5.0000514800514706E-2</v>
@@ -6095,7 +6094,7 @@
         <v>38504</v>
       </c>
       <c r="U71" s="15">
-        <v>47543</v>
+        <v>47542</v>
       </c>
       <c r="V71" s="12">
         <v>0</v>
@@ -6125,10 +6124,10 @@
         <v>5</v>
       </c>
       <c r="G72" s="15">
-        <v>47179</v>
+        <v>47178</v>
       </c>
       <c r="H72" s="15">
-        <v>47543</v>
+        <v>47542</v>
       </c>
       <c r="I72" s="9">
         <v>4.9999362628246669E-2</v>
@@ -6167,7 +6166,7 @@
         <v>38504</v>
       </c>
       <c r="U72" s="15">
-        <v>47543</v>
+        <v>47542</v>
       </c>
       <c r="V72" s="12">
         <v>0</v>
@@ -11092,10 +11091,10 @@
       <c r="F141" s="6">
         <v>2</v>
       </c>
-      <c r="G141" s="15">
+      <c r="G141" s="36">
         <v>45078</v>
       </c>
-      <c r="H141" s="15">
+      <c r="H141" s="36">
         <v>45443</v>
       </c>
       <c r="I141" s="9">
@@ -11164,10 +11163,10 @@
       <c r="F142" s="6">
         <v>3</v>
       </c>
-      <c r="G142" s="15">
+      <c r="G142" s="36">
         <v>45444</v>
       </c>
-      <c r="H142" s="15">
+      <c r="H142" s="36">
         <v>45808</v>
       </c>
       <c r="I142" s="9">
@@ -11236,10 +11235,10 @@
       <c r="F143" s="6">
         <v>4</v>
       </c>
-      <c r="G143" s="15">
+      <c r="G143" s="36">
         <v>45809</v>
       </c>
-      <c r="H143" s="15">
+      <c r="H143" s="36">
         <v>46173</v>
       </c>
       <c r="I143" s="9">
@@ -11308,10 +11307,10 @@
       <c r="F144" s="6">
         <v>5</v>
       </c>
-      <c r="G144" s="15">
+      <c r="G144" s="36">
         <v>46174</v>
       </c>
-      <c r="H144" s="15">
+      <c r="H144" s="36">
         <v>46538</v>
       </c>
       <c r="I144" s="9">
@@ -11741,10 +11740,10 @@
       <c r="F150" s="6">
         <v>5</v>
       </c>
-      <c r="G150" s="36">
+      <c r="G150" s="15">
         <v>46692</v>
       </c>
-      <c r="H150" s="36">
+      <c r="H150" s="15">
         <v>46706</v>
       </c>
       <c r="I150" s="9">
@@ -15846,7 +15845,7 @@
       <c r="G207" s="15">
         <v>46661</v>
       </c>
-      <c r="H207" s="36">
+      <c r="H207" s="15">
         <v>46810</v>
       </c>
       <c r="I207" s="9">
@@ -15919,7 +15918,7 @@
         <v>46811</v>
       </c>
       <c r="H208" s="39">
-        <v>47176</v>
+        <v>47177</v>
       </c>
       <c r="I208" s="40">
         <v>3.0174399212185676E-2</v>
@@ -15988,10 +15987,10 @@
         <v>8</v>
       </c>
       <c r="G209" s="39">
-        <v>47177</v>
+        <v>47178</v>
       </c>
       <c r="H209" s="39">
-        <v>47541</v>
+        <v>47542</v>
       </c>
       <c r="I209" s="40">
         <v>2.9829290206648595E-2</v>
@@ -16060,10 +16059,10 @@
         <v>9</v>
       </c>
       <c r="G210" s="39">
-        <v>47542</v>
+        <v>47543</v>
       </c>
       <c r="H210" s="39">
-        <v>47906</v>
+        <v>47907</v>
       </c>
       <c r="I210" s="40">
         <v>3.0012214273250848E-2</v>
@@ -16132,10 +16131,10 @@
         <v>10</v>
       </c>
       <c r="G211" s="39">
-        <v>47907</v>
+        <v>47908</v>
       </c>
       <c r="H211" s="39">
-        <v>48271</v>
+        <v>48273</v>
       </c>
       <c r="I211" s="40">
         <v>2.9984753515161611E-2</v>
@@ -16204,10 +16203,10 @@
         <v>11</v>
       </c>
       <c r="G212" s="39">
-        <v>48272</v>
+        <v>48274</v>
       </c>
       <c r="H212" s="39">
-        <v>48637</v>
+        <v>48638</v>
       </c>
       <c r="I212" s="40">
         <v>3.0098684210526416E-2</v>
@@ -16276,10 +16275,10 @@
         <v>12</v>
       </c>
       <c r="G213" s="44">
-        <v>48638</v>
+        <v>48639</v>
       </c>
       <c r="H213" s="44">
-        <v>49002</v>
+        <v>49003</v>
       </c>
       <c r="I213" s="45">
         <v>2.0000000000000018E-2</v>
@@ -16348,10 +16347,10 @@
         <v>13</v>
       </c>
       <c r="G214" s="44">
-        <v>49003</v>
+        <v>49004</v>
       </c>
       <c r="H214" s="44">
-        <v>49367</v>
+        <v>49368</v>
       </c>
       <c r="I214" s="45">
         <v>2.0000000000000018E-2</v>
@@ -16420,10 +16419,10 @@
         <v>14</v>
       </c>
       <c r="G215" s="44">
-        <v>49368</v>
+        <v>49369</v>
       </c>
       <c r="H215" s="44">
-        <v>49732</v>
+        <v>49734</v>
       </c>
       <c r="I215" s="45">
         <v>2.0000000000000018E-2</v>
@@ -16492,10 +16491,10 @@
         <v>15</v>
       </c>
       <c r="G216" s="44">
-        <v>49733</v>
+        <v>49735</v>
       </c>
       <c r="H216" s="44">
-        <v>50098</v>
+        <v>50099</v>
       </c>
       <c r="I216" s="45">
         <v>2.0000000000000018E-2</v>
@@ -16564,10 +16563,10 @@
         <v>16</v>
       </c>
       <c r="G217" s="44">
-        <v>50099</v>
+        <v>50100</v>
       </c>
       <c r="H217" s="44">
-        <v>50463</v>
+        <v>50464</v>
       </c>
       <c r="I217" s="45">
         <v>2.0000000000000018E-2</v>
@@ -18003,10 +18002,10 @@
       <c r="F237" s="6">
         <v>1</v>
       </c>
-      <c r="G237" s="59">
+      <c r="G237" s="36">
         <v>46158</v>
       </c>
-      <c r="H237" s="59">
+      <c r="H237" s="36">
         <v>46158</v>
       </c>
       <c r="I237" s="9">
@@ -18795,10 +18794,10 @@
       <c r="F248" s="6">
         <v>1</v>
       </c>
-      <c r="G248" s="15">
+      <c r="G248" s="36">
         <v>46143</v>
       </c>
-      <c r="H248" s="15">
+      <c r="H248" s="36">
         <v>46507</v>
       </c>
       <c r="I248" s="9">
@@ -18843,7 +18842,7 @@
       <c r="V248" s="12">
         <v>0</v>
       </c>
-      <c r="W248" s="60">
+      <c r="W248" s="59">
         <v>46417</v>
       </c>
       <c r="Z248" s="4"/>
@@ -18869,10 +18868,10 @@
       <c r="F249" s="6">
         <v>1</v>
       </c>
-      <c r="G249" s="15">
+      <c r="G249" s="36">
         <v>46508</v>
       </c>
-      <c r="H249" s="15">
+      <c r="H249" s="36">
         <v>46873</v>
       </c>
       <c r="I249" s="9">
@@ -18917,7 +18916,7 @@
       <c r="V249" s="12">
         <v>0</v>
       </c>
-      <c r="W249" s="60">
+      <c r="W249" s="59">
         <v>46783</v>
       </c>
       <c r="Z249" s="4"/>
@@ -18943,10 +18942,10 @@
       <c r="F250" s="6">
         <v>1</v>
       </c>
-      <c r="G250" s="15">
+      <c r="G250" s="36">
         <v>46874</v>
       </c>
-      <c r="H250" s="15">
+      <c r="H250" s="36">
         <v>47238</v>
       </c>
       <c r="I250" s="9">
@@ -18991,7 +18990,7 @@
       <c r="V250" s="12">
         <v>0</v>
       </c>
-      <c r="W250" s="60">
+      <c r="W250" s="59">
         <v>47148</v>
       </c>
       <c r="Z250" s="4"/>
@@ -19017,10 +19016,10 @@
       <c r="F251" s="6">
         <v>1</v>
       </c>
-      <c r="G251" s="15">
+      <c r="G251" s="36">
         <v>47239</v>
       </c>
-      <c r="H251" s="15">
+      <c r="H251" s="36">
         <v>47603</v>
       </c>
       <c r="I251" s="9">
@@ -19065,7 +19064,7 @@
       <c r="V251" s="12">
         <v>0</v>
       </c>
-      <c r="W251" s="60">
+      <c r="W251" s="59">
         <v>47513</v>
       </c>
       <c r="Z251" s="4"/>
@@ -19091,10 +19090,10 @@
       <c r="F252" s="6">
         <v>1</v>
       </c>
-      <c r="G252" s="15">
+      <c r="G252" s="36">
         <v>47604</v>
       </c>
-      <c r="H252" s="15">
+      <c r="H252" s="36">
         <v>47968</v>
       </c>
       <c r="I252" s="9">
@@ -19139,7 +19138,7 @@
       <c r="V252" s="12">
         <v>0</v>
       </c>
-      <c r="W252" s="60">
+      <c r="W252" s="59">
         <v>47878</v>
       </c>
       <c r="Z252" s="4"/>

</xml_diff>

<commit_message>
Dashboard update Mon 06/01/2026  9:15
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8745BF2F-DDBA-49AD-BFD6-931CA14D35B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{57E11860-C566-4DF6-B426-9CF179C4981F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2505" windowWidth="102195" windowHeight="29895" xr2:uid="{91136297-5822-44C6-A3F2-6CC3985E9C67}"/>
+    <workbookView xWindow="0" yWindow="2505" windowWidth="102195" windowHeight="29895" xr2:uid="{22111DD6-099B-4E7E-9EFF-4B98D6E63F34}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1919" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1918" uniqueCount="227">
   <si>
     <t>Building</t>
   </si>
@@ -461,7 +461,7 @@
     <t>Four (4) x 5-year AUTO-RENEWALS (no notice needed)</t>
   </si>
   <si>
-    <t>Annual termination on any anniversary w/ 90 days</t>
+    <t>Ann Anniversary w/ 90 days</t>
   </si>
   <si>
     <t>Electric Meter</t>
@@ -1282,7 +1282,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C57F37A-D4FD-4926-86E8-D42A75076906}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4FE9E19-F5EE-4DE3-BBD6-0D8558D90B59}">
   <dimension ref="A1:AT261"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -3887,9 +3887,7 @@
         <v>139</v>
       </c>
       <c r="AJ31" s="23"/>
-      <c r="AK31" s="20" t="s">
-        <v>140</v>
-      </c>
+      <c r="AK31" s="20"/>
       <c r="AL31" s="20" t="s">
         <v>140</v>
       </c>

</xml_diff>

<commit_message>
Dashboard update Wed 06/10/2026 22:01
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{57E11860-C566-4DF6-B426-9CF179C4981F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7921047B-9B90-4DB1-9D65-C4898713F0FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2505" windowWidth="102195" windowHeight="29895" xr2:uid="{22111DD6-099B-4E7E-9EFF-4B98D6E63F34}"/>
+    <workbookView xWindow="1380" yWindow="1290" windowWidth="50955" windowHeight="29895" xr2:uid="{4C8F54F5-FFF3-4038-96C5-A3C180D4E153}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1282,7 +1282,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4FE9E19-F5EE-4DE3-BBD6-0D8558D90B59}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC4E9431-E7F0-4412-A681-A0B0B0CD3550}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AT261"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -2478,13 +2479,13 @@
         <v>-10.571254319983737</v>
       </c>
       <c r="W18" s="16">
-        <v>46174</v>
+        <v>46182</v>
       </c>
       <c r="X18" s="16">
-        <v>46174</v>
+        <v>46182</v>
       </c>
       <c r="Y18" s="16">
-        <v>46174</v>
+        <v>46182</v>
       </c>
       <c r="Z18" s="17"/>
       <c r="AA18" s="18"/>
@@ -18764,10 +18765,10 @@
         <v>1</v>
       </c>
       <c r="G237" s="40">
-        <v>46174</v>
+        <v>46182</v>
       </c>
       <c r="H237" s="40">
-        <v>46174</v>
+        <v>46182</v>
       </c>
       <c r="I237" s="10">
         <v>0</v>
@@ -18800,13 +18801,13 @@
         <v>0</v>
       </c>
       <c r="S237" s="40">
-        <v>46174</v>
+        <v>46182</v>
       </c>
       <c r="T237" s="40">
-        <v>46174</v>
+        <v>46182</v>
       </c>
       <c r="U237" s="40">
-        <v>46174</v>
+        <v>46182</v>
       </c>
       <c r="V237" s="13">
         <v>0</v>

</xml_diff>

<commit_message>
Dashboard update Thu 06/11/2026 22:01
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7921047B-9B90-4DB1-9D65-C4898713F0FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{13E2EB8D-AD26-4432-9A11-07F6835F740E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1380" yWindow="1290" windowWidth="50955" windowHeight="29895" xr2:uid="{4C8F54F5-FFF3-4038-96C5-A3C180D4E153}"/>
+    <workbookView xWindow="2730" yWindow="1470" windowWidth="50955" windowHeight="29895" xr2:uid="{0E71905A-5A3E-47C2-A5C0-D077A0F4413D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1282,7 +1282,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC4E9431-E7F0-4412-A681-A0B0B0CD3550}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1380F1F3-91D5-4501-B71E-49695EF212CD}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AT261"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2479,13 +2479,13 @@
         <v>-10.571254319983737</v>
       </c>
       <c r="W18" s="16">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="X18" s="16">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="Y18" s="16">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="Z18" s="17"/>
       <c r="AA18" s="18"/>
@@ -18765,10 +18765,10 @@
         <v>1</v>
       </c>
       <c r="G237" s="40">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="H237" s="40">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="I237" s="10">
         <v>0</v>
@@ -18801,13 +18801,13 @@
         <v>0</v>
       </c>
       <c r="S237" s="40">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="T237" s="40">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="U237" s="40">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="V237" s="13">
         <v>0</v>

</xml_diff>

<commit_message>
Dashboard update Sat 08/22/2026  7:46
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2EA2EF8C-B10F-440D-B3B5-0FE2AB8AB47B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1F7E56E-72B5-429C-A408-4449914A8988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2025" yWindow="1170" windowWidth="52665" windowHeight="29925" xr2:uid="{92DBAD3C-EEC5-4140-B380-777927B5ED34}"/>
+    <workbookView xWindow="1770" yWindow="825" windowWidth="55830" windowHeight="31575" xr2:uid="{2343475C-3A1E-46A0-A498-F63CD467A17F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1361,7 +1361,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{637CCEBB-4FD6-486F-9E2D-6DA576487E5B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B22CD9-737D-43B8-B147-104813946A5C}">
   <dimension ref="A1:AT299"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -22349,10 +22349,10 @@
         <v>0</v>
       </c>
       <c r="J274" s="13">
-        <v>875</v>
+        <v>1500</v>
       </c>
       <c r="K274" s="56">
-        <v>10500</v>
+        <v>18000</v>
       </c>
       <c r="L274" s="6" t="s">
         <v>27</v>
@@ -22370,7 +22370,7 @@
         <v>3.9845497052246395E-2</v>
       </c>
       <c r="Q274" s="13">
-        <v>21.428571428571427</v>
+        <v>36.734693877551024</v>
       </c>
       <c r="R274" s="45">
         <v>2800</v>
@@ -22421,13 +22421,13 @@
         <v>46203</v>
       </c>
       <c r="I275" s="10">
-        <v>2.857142857142847E-2</v>
+        <v>3.3333333333333437E-2</v>
       </c>
       <c r="J275" s="13">
-        <v>900</v>
+        <v>1550</v>
       </c>
       <c r="K275" s="56">
-        <v>10800</v>
+        <v>18600</v>
       </c>
       <c r="L275" s="6" t="s">
         <v>27</v>
@@ -22445,7 +22445,7 @@
         <v>3.9845497052246395E-2</v>
       </c>
       <c r="Q275" s="13">
-        <v>22.040816326530614</v>
+        <v>37.95918367346939</v>
       </c>
       <c r="R275" s="45">
         <v>2800</v>
@@ -22496,13 +22496,13 @@
         <v>46568</v>
       </c>
       <c r="I276" s="10">
-        <v>2.7777777777777679E-2</v>
+        <v>3.2258064516129004E-2</v>
       </c>
       <c r="J276" s="13">
-        <v>925</v>
+        <v>1600</v>
       </c>
       <c r="K276" s="56">
-        <v>11100</v>
+        <v>19200</v>
       </c>
       <c r="L276" s="6" t="s">
         <v>27</v>
@@ -22520,7 +22520,7 @@
         <v>3.9845497052246395E-2</v>
       </c>
       <c r="Q276" s="13">
-        <v>22.653061224489797</v>
+        <v>39.183673469387756</v>
       </c>
       <c r="R276" s="45">
         <v>2800</v>
@@ -22647,10 +22647,10 @@
         <v>0</v>
       </c>
       <c r="J278" s="13">
-        <v>625</v>
+        <v>0</v>
       </c>
       <c r="K278" s="56">
-        <v>7500</v>
+        <v>0</v>
       </c>
       <c r="L278" s="6" t="s">
         <v>27</v>
@@ -22668,7 +22668,7 @@
         <v>2.2362268753811754E-2</v>
       </c>
       <c r="Q278" s="13">
-        <v>27.272727272727273</v>
+        <v>0</v>
       </c>
       <c r="R278" s="13">
         <v>0</v>
@@ -22718,14 +22718,14 @@
       <c r="H279" s="16">
         <v>46203</v>
       </c>
-      <c r="I279" s="10">
-        <v>4.0000000000000036E-2</v>
+      <c r="I279" s="10" t="e">
+        <v>#DIV/0!</v>
       </c>
       <c r="J279" s="13">
-        <v>650</v>
+        <v>0</v>
       </c>
       <c r="K279" s="56">
-        <v>7800</v>
+        <v>0</v>
       </c>
       <c r="L279" s="6" t="s">
         <v>27</v>
@@ -22743,7 +22743,7 @@
         <v>2.2362268753811754E-2</v>
       </c>
       <c r="Q279" s="13">
-        <v>28.363636363636363</v>
+        <v>0</v>
       </c>
       <c r="R279" s="13">
         <v>0</v>
@@ -22793,14 +22793,14 @@
       <c r="H280" s="16">
         <v>46568</v>
       </c>
-      <c r="I280" s="10">
-        <v>3.8461538461538547E-2</v>
+      <c r="I280" s="10" t="e">
+        <v>#DIV/0!</v>
       </c>
       <c r="J280" s="13">
-        <v>675</v>
+        <v>0</v>
       </c>
       <c r="K280" s="56">
-        <v>8100</v>
+        <v>0</v>
       </c>
       <c r="L280" s="6" t="s">
         <v>27</v>
@@ -22818,7 +22818,7 @@
         <v>2.2362268753811754E-2</v>
       </c>
       <c r="Q280" s="13">
-        <v>29.454545454545453</v>
+        <v>0</v>
       </c>
       <c r="R280" s="13">
         <v>0</v>

</xml_diff>

<commit_message>
Dashboard update Sat 08/22/2026 11:08
</commit_message>
<xml_diff>
--- a/data/MSP Tenancy.xlsx
+++ b/data/MSP Tenancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\OpenClaw\Share Jason\General Procedures\msp-dashboard-src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1F7E56E-72B5-429C-A408-4449914A8988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A01070D5-8645-4D4B-B525-6E0C5E48D612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1770" yWindow="825" windowWidth="55830" windowHeight="31575" xr2:uid="{2343475C-3A1E-46A0-A498-F63CD467A17F}"/>
+    <workbookView xWindow="1770" yWindow="825" windowWidth="55830" windowHeight="31575" xr2:uid="{ACF3E97C-5406-46E4-9E78-276C232D0021}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1361,7 +1361,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B22CD9-737D-43B8-B147-104813946A5C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50AC4753-2301-471E-B36E-F3CC99F16AFA}">
   <dimension ref="A1:AT299"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -16325,10 +16325,10 @@
         <v>0</v>
       </c>
       <c r="J194" s="13">
-        <v>1</v>
+        <v>2600</v>
       </c>
       <c r="K194" s="56">
-        <v>12</v>
+        <v>31200</v>
       </c>
       <c r="L194" s="6" t="s">
         <v>36</v>
@@ -16346,10 +16346,10 @@
         <v>0</v>
       </c>
       <c r="Q194" s="13">
-        <v>9.3312597200622092E-3</v>
+        <v>24.261275272161743</v>
       </c>
       <c r="R194" s="13">
-        <v>1.5</v>
+        <v>3900</v>
       </c>
       <c r="S194" s="43">
         <v>46249</v>
@@ -20331,13 +20331,13 @@
         <v>46599</v>
       </c>
       <c r="I247" s="10">
-        <v>5.0000000000000044E-2</v>
+        <v>4.9886621315192725E-2</v>
       </c>
       <c r="J247" s="13">
-        <v>4630.5</v>
+        <v>4630</v>
       </c>
       <c r="K247" s="56">
-        <v>55566</v>
+        <v>55560</v>
       </c>
       <c r="L247" s="6" t="s">
         <v>56</v>
@@ -20355,7 +20355,7 @@
         <v>0.1741</v>
       </c>
       <c r="Q247" s="13">
-        <v>38.694986072423397</v>
+        <v>38.690807799442894</v>
       </c>
       <c r="R247" s="45">
         <v>3000</v>
@@ -20409,10 +20409,10 @@
         <v>0</v>
       </c>
       <c r="J248" s="13">
-        <v>4630.5</v>
+        <v>4630</v>
       </c>
       <c r="K248" s="56">
-        <v>55566</v>
+        <v>55560</v>
       </c>
       <c r="L248" s="6" t="s">
         <v>56</v>
@@ -20430,7 +20430,7 @@
         <v>0.1741</v>
       </c>
       <c r="Q248" s="13">
-        <v>38.694986072423397</v>
+        <v>38.690807799442894</v>
       </c>
       <c r="R248" s="45">
         <v>3000</v>
@@ -20484,10 +20484,10 @@
         <v>0</v>
       </c>
       <c r="J249" s="13">
-        <v>4630.5</v>
+        <v>4630</v>
       </c>
       <c r="K249" s="56">
-        <v>55566</v>
+        <v>55560</v>
       </c>
       <c r="L249" s="6" t="s">
         <v>56</v>
@@ -20505,7 +20505,7 @@
         <v>0.1741</v>
       </c>
       <c r="Q249" s="13">
-        <v>38.694986072423397</v>
+        <v>38.690807799442894</v>
       </c>
       <c r="R249" s="45">
         <v>3000</v>
@@ -21474,8 +21474,8 @@
       <c r="Q262" s="13">
         <v>0</v>
       </c>
-      <c r="R262" s="13">
-        <v>0</v>
+      <c r="R262" s="56">
+        <v>4800</v>
       </c>
       <c r="S262" s="43">
         <v>46235</v>
@@ -23501,8 +23501,8 @@
       <c r="Q289" s="13">
         <v>17.402269861286253</v>
       </c>
-      <c r="R289" s="13">
-        <v>0</v>
+      <c r="R289" s="56">
+        <v>1700</v>
       </c>
       <c r="S289" s="43">
         <v>39520</v>

</xml_diff>